<commit_message>
LUPA: siembra las compras fraccionadas y quita el contador del titular
El caso de las seis ordenes de compra bajo el umbral no estaba en los
datos, asi que R11 solo veia ruido; ahora esta sembrado y la regla lo
encuentra como un unico hallazgo. El motor ajusta el reparto del monto
por documento y la banda superior se queda sin la cifra gigante, que
se desbordaba de su caja.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel Distribuidora Andina/01 Terceros.xlsx
+++ b/Excel Distribuidora Andina/01 Terceros.xlsx
@@ -455,22 +455,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D2" t="str">
-        <v>851.787.205-8</v>
+        <v>818.697.317-8</v>
       </c>
       <c r="E2" t="str">
-        <v>604 477 89 97</v>
+        <v>604 466 88 47</v>
       </c>
       <c r="F2" t="str">
-        <v>Transversal 89A # 47 - 96, El Poblado, Medellín</v>
+        <v>Calle 79 # 98 - 86, Laureles, Medellín</v>
       </c>
       <c r="G2" t="str">
-        <v>6629142994</v>
+        <v>2907529516</v>
       </c>
       <c r="H2" t="str">
-        <v>BBVA Colombia</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I2" t="str">
-        <v>18/11/2023</v>
+        <v>11/10/2017</v>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -487,22 +487,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D3" t="str">
-        <v>836.209.170-6</v>
+        <v>832.979.170-4</v>
       </c>
       <c r="E3" t="str">
-        <v>604 690 53 79</v>
+        <v>604 223 32 96</v>
       </c>
       <c r="F3" t="str">
-        <v>Calle 96 # 55 - 85, Girardota, Medellín</v>
+        <v>Calle 72A # 91 - 58, La América, Medellín</v>
       </c>
       <c r="G3" t="str">
-        <v>7900835031</v>
+        <v>6651395333</v>
       </c>
       <c r="H3" t="str">
-        <v>Scotiabank Colpatria</v>
+        <v>Banco de Bogotá</v>
       </c>
       <c r="I3" t="str">
-        <v>06/08/2023</v>
+        <v>09/05/2023</v>
       </c>
       <c r="J3" t="str">
         <v>mosorio</v>
@@ -519,22 +519,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D4" t="str">
-        <v>837.200.419-7</v>
+        <v>896.209.534-1</v>
       </c>
       <c r="E4" t="str">
-        <v>604 681 23 19</v>
+        <v>604 563 73 71</v>
       </c>
       <c r="F4" t="str">
-        <v>Carrera 45 # 88 - 62, San Javier, Medellín</v>
+        <v>Avenida 95 # 95 - 30, San Javier, Medellín</v>
       </c>
       <c r="G4" t="str">
-        <v>3562781588</v>
+        <v>3398331476</v>
       </c>
       <c r="H4" t="str">
-        <v>Davivienda</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I4" t="str">
-        <v>28/11/2020</v>
+        <v>16/01/2020</v>
       </c>
       <c r="J4" t="str">
         <v/>
@@ -551,22 +551,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D5" t="str">
-        <v>801.894.972-5</v>
+        <v>846.232.835-8</v>
       </c>
       <c r="E5" t="str">
-        <v>604 583 68 74</v>
+        <v>604 361 25 23</v>
       </c>
       <c r="F5" t="str">
-        <v>Carrera 33 # 7 - 24, Itagüí, Medellín</v>
+        <v>Transversal 26 # 86 - 72, Bello, Medellín</v>
       </c>
       <c r="G5" t="str">
-        <v>4838044015</v>
+        <v>2506643589</v>
       </c>
       <c r="H5" t="str">
-        <v>Banco de Occidente</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I5" t="str">
-        <v>13/10/2018</v>
+        <v>04/09/2019</v>
       </c>
       <c r="J5" t="str">
         <v>mosorio</v>
@@ -583,25 +583,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D6" t="str">
-        <v>888.555.778-5</v>
+        <v>855.720.452-7</v>
       </c>
       <c r="E6" t="str">
-        <v>604 343 26 36</v>
+        <v>604 870 32 15</v>
       </c>
       <c r="F6" t="str">
-        <v>Carrera 10 # 67 - 18, Aranjuez, Medellín</v>
+        <v>Diagonal 1 # 80 - 67, Copacabana, Medellín</v>
       </c>
       <c r="G6" t="str">
-        <v>5104172701</v>
+        <v>3810095395</v>
       </c>
       <c r="H6" t="str">
-        <v>Scotiabank Colpatria</v>
+        <v>Banco de Bogotá</v>
       </c>
       <c r="I6" t="str">
-        <v>08/07/2018</v>
+        <v>22/05/2024</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="7">
@@ -615,22 +615,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D7" t="str">
-        <v>811.337.496-9</v>
+        <v>845.283.034-1</v>
       </c>
       <c r="E7" t="str">
-        <v>604 667 55 40</v>
+        <v>604 895 96 49</v>
       </c>
       <c r="F7" t="str">
-        <v>Diagonal 31 # 65 - 46, Manrique, Medellín</v>
+        <v>Avenida 58 # 33 - 69, Caldas, Medellín</v>
       </c>
       <c r="G7" t="str">
-        <v>1136986347</v>
+        <v>7411872399</v>
       </c>
       <c r="H7" t="str">
-        <v>Banco AV Villas</v>
+        <v>Banco de Occidente</v>
       </c>
       <c r="I7" t="str">
-        <v>03/01/2020</v>
+        <v>21/10/2021</v>
       </c>
       <c r="J7" t="str">
         <v>mosorio</v>
@@ -647,22 +647,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D8" t="str">
-        <v>871.732.178-3</v>
+        <v>895.320.346-3</v>
       </c>
       <c r="E8" t="str">
-        <v>604 623 87 83</v>
+        <v>604 424 65 52</v>
       </c>
       <c r="F8" t="str">
-        <v>Diagonal 78 # 48 - 49, Rionegro, Medellín</v>
+        <v>Diagonal 19A # 51 - 58, Aranjuez, Medellín</v>
       </c>
       <c r="G8" t="str">
-        <v>4526658046</v>
+        <v>6855349157</v>
       </c>
       <c r="H8" t="str">
-        <v>Itaú Colombia</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I8" t="str">
-        <v>10/02/2020</v>
+        <v>07/06/2018</v>
       </c>
       <c r="J8" t="str">
         <v>mosorio</v>
@@ -679,25 +679,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D9" t="str">
-        <v>873.382.518-9</v>
+        <v>854.169.427-6</v>
       </c>
       <c r="E9" t="str">
-        <v>604 402 79 77</v>
+        <v>604 898 34 12</v>
       </c>
       <c r="F9" t="str">
-        <v>Calle 10 # 39 - 87, Laureles, Medellín</v>
+        <v>Calle 85 # 62 - 74, Robledo, Medellín</v>
       </c>
       <c r="G9" t="str">
-        <v>7552307676</v>
+        <v>6154144469</v>
       </c>
       <c r="H9" t="str">
-        <v>Banco de Occidente</v>
+        <v>Banco de Bogotá</v>
       </c>
       <c r="I9" t="str">
-        <v>12/12/2016</v>
+        <v>21/05/2017</v>
       </c>
       <c r="J9" t="str">
-        <v>mosorio</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -711,22 +711,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D10" t="str">
-        <v>811.706.637-4</v>
+        <v>860.122.973-5</v>
       </c>
       <c r="E10" t="str">
-        <v>604 734 91 84</v>
+        <v>604 210 72 73</v>
       </c>
       <c r="F10" t="str">
-        <v>Calle 30 # 68 - 37, Buenos Aires, Medellín</v>
+        <v>Carrera 21 # 99 - 44, Manrique, Medellín</v>
       </c>
       <c r="G10" t="str">
-        <v>5535232466</v>
+        <v>2112400636</v>
       </c>
       <c r="H10" t="str">
-        <v>Banco Agrario de Colombia</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I10" t="str">
-        <v>14/10/2021</v>
+        <v>27/04/2017</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -743,25 +743,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D11" t="str">
-        <v>868.081.661-4</v>
+        <v>807.476.911-5</v>
       </c>
       <c r="E11" t="str">
-        <v>604 657 24 28</v>
+        <v>604 782 33 53</v>
       </c>
       <c r="F11" t="str">
-        <v>Transversal 64 # 72 - 83, La América, Medellín</v>
+        <v>Carrera 65 # 39 - 85, Envigado, Medellín</v>
       </c>
       <c r="G11" t="str">
-        <v>3790585374</v>
+        <v>1711535493</v>
       </c>
       <c r="H11" t="str">
-        <v>Banco AV Villas</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I11" t="str">
-        <v>05/11/2024</v>
+        <v>08/12/2023</v>
       </c>
       <c r="J11" t="str">
-        <v>mosorio</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -775,22 +775,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D12" t="str">
-        <v>878.235.290-4</v>
+        <v>820.908.830-1</v>
       </c>
       <c r="E12" t="str">
-        <v>604 661 70 90</v>
+        <v>604 704 58 78</v>
       </c>
       <c r="F12" t="str">
-        <v>Diagonal 34 # 88 - 18, Manrique, Medellín</v>
+        <v>Calle 61 # 42 - 91, San Javier, Medellín</v>
       </c>
       <c r="G12" t="str">
-        <v>5520362592</v>
+        <v>7823257628</v>
       </c>
       <c r="H12" t="str">
-        <v>Banco de Bogotá</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I12" t="str">
-        <v>10/03/2024</v>
+        <v>24/02/2021</v>
       </c>
       <c r="J12" t="str">
         <v>mosorio</v>
@@ -807,25 +807,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D13" t="str">
-        <v>839.956.672-6</v>
+        <v>864.856.423-0</v>
       </c>
       <c r="E13" t="str">
-        <v>604 250 77 68</v>
+        <v>604 460 14 63</v>
       </c>
       <c r="F13" t="str">
-        <v>Carrera 28 # 97 - 55, Castilla, Medellín</v>
+        <v>Avenida 36 # 79 - 93, La Estrella, Medellín</v>
       </c>
       <c r="G13" t="str">
-        <v>2568516855</v>
+        <v>7118761020</v>
       </c>
       <c r="H13" t="str">
-        <v>Banco de Bogotá</v>
+        <v>Banco Agrario de Colombia</v>
       </c>
       <c r="I13" t="str">
-        <v>31/12/2016</v>
+        <v>14/07/2021</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="14">
@@ -839,22 +839,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D14" t="str">
-        <v>874.983.880-3</v>
+        <v>812.789.772-1</v>
       </c>
       <c r="E14" t="str">
-        <v>604 331 89 45</v>
+        <v>604 654 39 59</v>
       </c>
       <c r="F14" t="str">
-        <v>Transversal 6 # 96 - 66, Itagüí, Medellín</v>
+        <v>Calle 87 # 17 - 22, San Javier, Medellín</v>
       </c>
       <c r="G14" t="str">
-        <v>3719334233</v>
+        <v>5931742714</v>
       </c>
       <c r="H14" t="str">
-        <v>Banco de Bogotá</v>
+        <v>Banco de Occidente</v>
       </c>
       <c r="I14" t="str">
-        <v>11/07/2018</v>
+        <v>04/07/2023</v>
       </c>
       <c r="J14" t="str">
         <v>mosorio</v>
@@ -871,22 +871,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D15" t="str">
-        <v>830.769.676-0</v>
+        <v>868.096.302-0</v>
       </c>
       <c r="E15" t="str">
-        <v>604 283 67 59</v>
+        <v>604 544 59 64</v>
       </c>
       <c r="F15" t="str">
-        <v>Avenida 74 # 65 - 61, Sabaneta, Medellín</v>
+        <v>Carrera 90 # 68 - 81, Guayabal, Medellín</v>
       </c>
       <c r="G15" t="str">
-        <v>1931346847</v>
+        <v>3228709798</v>
       </c>
       <c r="H15" t="str">
-        <v>Scotiabank Colpatria</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I15" t="str">
-        <v>25/03/2017</v>
+        <v>18/07/2021</v>
       </c>
       <c r="J15" t="str">
         <v>mosorio</v>
@@ -903,22 +903,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D16" t="str">
-        <v>839.273.050-3</v>
+        <v>888.141.520-5</v>
       </c>
       <c r="E16" t="str">
-        <v>604 453 13 58</v>
+        <v>604 896 61 74</v>
       </c>
       <c r="F16" t="str">
-        <v>Transversal 32 # 48 - 60, Girardota, Medellín</v>
+        <v>Calle 64 # 64 - 77, El Poblado, Medellín</v>
       </c>
       <c r="G16" t="str">
-        <v>2289480539</v>
+        <v>6888822079</v>
       </c>
       <c r="H16" t="str">
-        <v>Itaú Colombia</v>
+        <v>Banco de Occidente</v>
       </c>
       <c r="I16" t="str">
-        <v>14/01/2022</v>
+        <v>21/06/2018</v>
       </c>
       <c r="J16" t="str">
         <v/>
@@ -935,22 +935,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D17" t="str">
-        <v>816.097.272-3</v>
+        <v>810.255.943-3</v>
       </c>
       <c r="E17" t="str">
-        <v>604 633 57 65</v>
+        <v>604 860 83 72</v>
       </c>
       <c r="F17" t="str">
-        <v>Calle 80 # 40 - 71, Itagüí, Medellín</v>
+        <v>Diagonal 90 # 16 - 60, Rionegro, Medellín</v>
       </c>
       <c r="G17" t="str">
-        <v>3924700136</v>
+        <v>5560424656</v>
       </c>
       <c r="H17" t="str">
-        <v>Bancolombia</v>
+        <v>Davivienda</v>
       </c>
       <c r="I17" t="str">
-        <v>23/05/2020</v>
+        <v>14/06/2018</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -967,25 +967,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D18" t="str">
-        <v>849.453.361-8</v>
+        <v>828.349.073-0</v>
       </c>
       <c r="E18" t="str">
-        <v>604 214 50 55</v>
+        <v>604 620 98 34</v>
       </c>
       <c r="F18" t="str">
-        <v>Diagonal 22A # 67 - 34, La Estrella, Medellín</v>
+        <v>Diagonal 88 # 43 - 53, Laureles, Medellín</v>
       </c>
       <c r="G18" t="str">
-        <v>1675310217</v>
+        <v>4679142465</v>
       </c>
       <c r="H18" t="str">
-        <v>Banco de Occidente</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I18" t="str">
-        <v>05/03/2018</v>
+        <v>31/12/2020</v>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="19">
@@ -999,22 +999,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D19" t="str">
-        <v>871.400.553-8</v>
+        <v>866.459.159-5</v>
       </c>
       <c r="E19" t="str">
-        <v>604 413 38 99</v>
+        <v>604 528 52 39</v>
       </c>
       <c r="F19" t="str">
-        <v>Calle 90 # 87 - 95, La Estrella, Medellín</v>
+        <v>Transversal 60 # 50 - 33, El Poblado, Medellín</v>
       </c>
       <c r="G19" t="str">
-        <v>9189554741</v>
+        <v>9853876568</v>
       </c>
       <c r="H19" t="str">
-        <v>Banco AV Villas</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I19" t="str">
-        <v>25/08/2021</v>
+        <v>14/05/2021</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -1031,25 +1031,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D20" t="str">
-        <v>823.814.662-5</v>
+        <v>873.226.766-1</v>
       </c>
       <c r="E20" t="str">
-        <v>604 212 15 42</v>
+        <v>604 287 27 67</v>
       </c>
       <c r="F20" t="str">
-        <v>Calle 97 # 49 - 28, Bello, Medellín</v>
+        <v>Carrera 56 # 17 - 43, Envigado, Medellín</v>
       </c>
       <c r="G20" t="str">
-        <v>6183049130</v>
+        <v>1839009313</v>
       </c>
       <c r="H20" t="str">
-        <v>Bancolombia</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I20" t="str">
-        <v>21/08/2016</v>
+        <v>30/03/2024</v>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="21">
@@ -1063,22 +1063,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D21" t="str">
-        <v>852.307.623-9</v>
+        <v>879.945.696-0</v>
       </c>
       <c r="E21" t="str">
-        <v>604 648 85 11</v>
+        <v>604 875 89 51</v>
       </c>
       <c r="F21" t="str">
-        <v>Calle 23 # 58 - 76, Itagüí, Medellín</v>
+        <v>Calle 2 # 74 - 76, Itagüí, Medellín</v>
       </c>
       <c r="G21" t="str">
-        <v>5724539224</v>
+        <v>4865957610</v>
       </c>
       <c r="H21" t="str">
         <v>Scotiabank Colpatria</v>
       </c>
       <c r="I21" t="str">
-        <v>28/02/2017</v>
+        <v>16/10/2017</v>
       </c>
       <c r="J21" t="str">
         <v>mosorio</v>
@@ -1095,22 +1095,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D22" t="str">
-        <v>878.012.093-2</v>
+        <v>804.394.891-2</v>
       </c>
       <c r="E22" t="str">
-        <v>604 203 88 46</v>
+        <v>604 331 65 61</v>
       </c>
       <c r="F22" t="str">
-        <v>Avenida 26 # 36 - 37, El Poblado, Medellín</v>
+        <v>Calle 76 # 41 - 33, Belén, Medellín</v>
       </c>
       <c r="G22" t="str">
-        <v>5389169069</v>
+        <v>8467756327</v>
       </c>
       <c r="H22" t="str">
-        <v>Davivienda</v>
+        <v>Banco AV Villas</v>
       </c>
       <c r="I22" t="str">
-        <v>19/07/2016</v>
+        <v>25/12/2021</v>
       </c>
       <c r="J22" t="str">
         <v>mosorio</v>
@@ -1127,22 +1127,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D23" t="str">
-        <v>888.825.902-1</v>
+        <v>828.630.464-0</v>
       </c>
       <c r="E23" t="str">
-        <v>604 756 89 52</v>
+        <v>604 560 17 44</v>
       </c>
       <c r="F23" t="str">
-        <v>Calle 44A # 17 - 44, Guayabal, Medellín</v>
+        <v>Avenida 24 # 70 - 90, San Javier, Medellín</v>
       </c>
       <c r="G23" t="str">
-        <v>4500439384</v>
+        <v>2728924112</v>
       </c>
       <c r="H23" t="str">
-        <v>BBVA Colombia</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I23" t="str">
-        <v>12/09/2017</v>
+        <v>13/08/2021</v>
       </c>
       <c r="J23" t="str">
         <v>mosorio</v>
@@ -1159,25 +1159,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D24" t="str">
-        <v>823.381.397-8</v>
+        <v>894.236.353-2</v>
       </c>
       <c r="E24" t="str">
-        <v>604 658 59 89</v>
+        <v>604 531 87 77</v>
       </c>
       <c r="F24" t="str">
-        <v>Transversal 26 # 78 - 41, Laureles, Medellín</v>
+        <v>Transversal 41 # 93 - 16, Girardota, Medellín</v>
       </c>
       <c r="G24" t="str">
-        <v>2796709053</v>
+        <v>3603789475</v>
       </c>
       <c r="H24" t="str">
-        <v>Banco AV Villas</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I24" t="str">
-        <v>06/01/2018</v>
+        <v>19/08/2019</v>
       </c>
       <c r="J24" t="str">
-        <v>mosorio</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1191,25 +1191,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D25" t="str">
-        <v>871.715.918-5</v>
+        <v>879.562.020-8</v>
       </c>
       <c r="E25" t="str">
-        <v>604 638 17 70</v>
+        <v>604 241 12 52</v>
       </c>
       <c r="F25" t="str">
-        <v>Carrera 82A # 22 - 75, La Estrella, Medellín</v>
+        <v>Calle 25 # 63 - 98, Laureles, Medellín</v>
       </c>
       <c r="G25" t="str">
-        <v>1711064599</v>
+        <v>2699477743</v>
       </c>
       <c r="H25" t="str">
-        <v>Itaú Colombia</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I25" t="str">
-        <v>23/11/2016</v>
+        <v>11/09/2023</v>
       </c>
       <c r="J25" t="str">
-        <v>mosorio</v>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1223,25 +1223,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D26" t="str">
-        <v>838.339.796-0</v>
+        <v>865.741.672-7</v>
       </c>
       <c r="E26" t="str">
-        <v>604 383 45 53</v>
+        <v>604 677 20 16</v>
       </c>
       <c r="F26" t="str">
-        <v>Avenida 37 # 18 - 96, Bello, Medellín</v>
+        <v>Transversal 51 # 88 - 97, Robledo, Medellín</v>
       </c>
       <c r="G26" t="str">
-        <v>1911285422</v>
+        <v>9234136214</v>
       </c>
       <c r="H26" t="str">
-        <v>Banco de Occidente</v>
+        <v>Banco Agrario de Colombia</v>
       </c>
       <c r="I26" t="str">
-        <v>13/04/2022</v>
+        <v>29/09/2016</v>
       </c>
       <c r="J26" t="str">
-        <v>mosorio</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1255,22 +1255,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D27" t="str">
-        <v>878.126.888-0</v>
+        <v>858.617.793-4</v>
       </c>
       <c r="E27" t="str">
-        <v>604 529 24 14</v>
+        <v>604 503 41 87</v>
       </c>
       <c r="F27" t="str">
-        <v>Calle 89 # 40 - 64, Girardota, Medellín</v>
+        <v>Diagonal 36 # 49 - 79, Laureles, Medellín</v>
       </c>
       <c r="G27" t="str">
-        <v>3913258427</v>
+        <v>9847318705</v>
       </c>
       <c r="H27" t="str">
-        <v>Itaú Colombia</v>
+        <v>Banco AV Villas</v>
       </c>
       <c r="I27" t="str">
-        <v>26/12/2021</v>
+        <v>12/05/2024</v>
       </c>
       <c r="J27" t="str">
         <v/>
@@ -1287,22 +1287,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D28" t="str">
-        <v>865.222.604-1</v>
+        <v>888.202.037-1</v>
       </c>
       <c r="E28" t="str">
-        <v>604 774 71 39</v>
+        <v>604 302 77 84</v>
       </c>
       <c r="F28" t="str">
-        <v>Carrera 47 # 45 - 83, Robledo, Medellín</v>
+        <v>Calle 37 # 16 - 19, Bello, Medellín</v>
       </c>
       <c r="G28" t="str">
-        <v>4554705809</v>
+        <v>5419761858</v>
       </c>
       <c r="H28" t="str">
-        <v>Banco Popular</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I28" t="str">
-        <v>15/09/2024</v>
+        <v>01/07/2022</v>
       </c>
       <c r="J28" t="str">
         <v>mosorio</v>
@@ -1319,25 +1319,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D29" t="str">
-        <v>831.637.287-6</v>
+        <v>851.391.773-9</v>
       </c>
       <c r="E29" t="str">
-        <v>604 790 90 24</v>
+        <v>604 803 19 56</v>
       </c>
       <c r="F29" t="str">
-        <v>Diagonal 6 # 6 - 19, Laureles, Medellín</v>
+        <v>Avenida 1 # 65 - 74, Sabaneta, Medellín</v>
       </c>
       <c r="G29" t="str">
-        <v>3771019889</v>
+        <v>4455155790</v>
       </c>
       <c r="H29" t="str">
-        <v>Banco Agrario de Colombia</v>
+        <v>Davivienda</v>
       </c>
       <c r="I29" t="str">
-        <v>24/03/2017</v>
+        <v>19/10/2018</v>
       </c>
       <c r="J29" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="30">
@@ -1351,25 +1351,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D30" t="str">
-        <v>831.181.945-5</v>
+        <v>881.364.793-0</v>
       </c>
       <c r="E30" t="str">
-        <v>604 758 34 70</v>
+        <v>604 575 46 34</v>
       </c>
       <c r="F30" t="str">
-        <v>Calle 45A # 19 - 16, Manrique, Medellín</v>
+        <v>Calle 88A # 19 - 36, Itagüí, Medellín</v>
       </c>
       <c r="G30" t="str">
-        <v>4996435594</v>
+        <v>1566607366</v>
       </c>
       <c r="H30" t="str">
-        <v>Banco AV Villas</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I30" t="str">
-        <v>09/06/2023</v>
+        <v>16/11/2021</v>
       </c>
       <c r="J30" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="31">
@@ -1383,25 +1383,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D31" t="str">
-        <v>849.766.232-1</v>
+        <v>801.454.360-0</v>
       </c>
       <c r="E31" t="str">
-        <v>604 216 61 33</v>
+        <v>604 319 74 31</v>
       </c>
       <c r="F31" t="str">
-        <v>Carrera 49 # 66 - 41, La América, Medellín</v>
+        <v>Avenida 11 # 50 - 40, San Javier, Medellín</v>
       </c>
       <c r="G31" t="str">
-        <v>2239744214</v>
+        <v>3967810916</v>
       </c>
       <c r="H31" t="str">
-        <v>Banco de Bogotá</v>
+        <v>Banco de Occidente</v>
       </c>
       <c r="I31" t="str">
-        <v>16/11/2016</v>
+        <v>04/03/2022</v>
       </c>
       <c r="J31" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="32">
@@ -1415,25 +1415,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D32" t="str">
-        <v>888.399.743-9</v>
+        <v>805.027.402-5</v>
       </c>
       <c r="E32" t="str">
-        <v>604 356 80 18</v>
+        <v>604 710 83 47</v>
       </c>
       <c r="F32" t="str">
-        <v>Calle 61 # 25 - 58, Caldas, Medellín</v>
+        <v>Carrera 71 # 85 - 83, Aranjuez, Medellín</v>
       </c>
       <c r="G32" t="str">
         <v>8801234455</v>
       </c>
       <c r="H32" t="str">
-        <v>Banco Popular</v>
+        <v>Banco de Occidente</v>
       </c>
       <c r="I32" t="str">
-        <v>09/02/2024</v>
+        <v>05/09/2024</v>
       </c>
       <c r="J32" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="33">
@@ -1447,25 +1447,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D33" t="str">
-        <v>857.498.355-6</v>
+        <v>847.458.320-1</v>
       </c>
       <c r="E33" t="str">
-        <v>604 262 11 58</v>
+        <v>604 640 55 48</v>
       </c>
       <c r="F33" t="str">
-        <v>Calle 38 # 96 - 74, Aranjuez, Medellín</v>
+        <v>Carrera 73 # 77 - 77, Guayabal, Medellín</v>
       </c>
       <c r="G33" t="str">
-        <v>6546377376</v>
+        <v>1442338783</v>
       </c>
       <c r="H33" t="str">
-        <v>Banco de Bogotá</v>
+        <v>Banco AV Villas</v>
       </c>
       <c r="I33" t="str">
-        <v>21/12/2017</v>
+        <v>04/04/2017</v>
       </c>
       <c r="J33" t="str">
-        <v>mosorio</v>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1479,22 +1479,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D34" t="str">
-        <v>843.253.718-3</v>
+        <v>850.251.281-3</v>
       </c>
       <c r="E34" t="str">
-        <v>604 209 96 40</v>
+        <v>604 648 53 15</v>
       </c>
       <c r="F34" t="str">
-        <v>Avenida 32A # 98 - 54, San Javier, Medellín</v>
+        <v>Transversal 11 # 90 - 84, El Poblado, Medellín</v>
       </c>
       <c r="G34" t="str">
-        <v>5183218254</v>
+        <v>3598561166</v>
       </c>
       <c r="H34" t="str">
-        <v>Banco AV Villas</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I34" t="str">
-        <v>07/10/2021</v>
+        <v>08/11/2020</v>
       </c>
       <c r="J34" t="str">
         <v>mosorio</v>
@@ -1511,22 +1511,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D35" t="str">
-        <v>808.393.964-1</v>
+        <v>848.391.980-6</v>
       </c>
       <c r="E35" t="str">
-        <v>604 403 62 74</v>
+        <v>604 667 93 66</v>
       </c>
       <c r="F35" t="str">
-        <v>Avenida 5 # 19 - 74, Sabaneta, Medellín</v>
+        <v>Diagonal 68 # 16 - 28, Robledo, Medellín</v>
       </c>
       <c r="G35" t="str">
-        <v>6280739002</v>
+        <v>6358929247</v>
       </c>
       <c r="H35" t="str">
         <v>Banco AV Villas</v>
       </c>
       <c r="I35" t="str">
-        <v>21/04/2022</v>
+        <v>24/04/2020</v>
       </c>
       <c r="J35" t="str">
         <v>mosorio</v>
@@ -1543,22 +1543,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D36" t="str">
-        <v>816.141.984-7</v>
+        <v>876.197.074-9</v>
       </c>
       <c r="E36" t="str">
-        <v>604 673 58 49</v>
+        <v>604 481 85 97</v>
       </c>
       <c r="F36" t="str">
-        <v>Carrera 63 # 64 - 11, San Javier, Medellín</v>
+        <v>Calle 78 # 67 - 90, Aranjuez, Medellín</v>
       </c>
       <c r="G36" t="str">
-        <v>4885996718</v>
+        <v>4841477328</v>
       </c>
       <c r="H36" t="str">
-        <v>Banco de Bogotá</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I36" t="str">
-        <v>11/07/2016</v>
+        <v>09/05/2022</v>
       </c>
       <c r="J36" t="str">
         <v>mosorio</v>
@@ -1575,22 +1575,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D37" t="str">
-        <v>850.660.833-3</v>
+        <v>846.772.816-4</v>
       </c>
       <c r="E37" t="str">
-        <v>604 708 92 81</v>
+        <v>604 340 33 91</v>
       </c>
       <c r="F37" t="str">
-        <v>Avenida 90 # 6 - 65, Bello, Medellín</v>
+        <v>Calle 39A # 74 - 68, Itagüí, Medellín</v>
       </c>
       <c r="G37" t="str">
-        <v>1774517955</v>
+        <v>3376575189</v>
       </c>
       <c r="H37" t="str">
-        <v>Scotiabank Colpatria</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I37" t="str">
-        <v>19/09/2022</v>
+        <v>19/06/2021</v>
       </c>
       <c r="J37" t="str">
         <v>mosorio</v>
@@ -1607,22 +1607,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D38" t="str">
-        <v>812.864.050-1</v>
+        <v>852.016.279-9</v>
       </c>
       <c r="E38" t="str">
-        <v>604 591 78 19</v>
+        <v>604 602 36 16</v>
       </c>
       <c r="F38" t="str">
-        <v>Diagonal 4 # 37 - 15, Copacabana, Medellín</v>
+        <v>Avenida 74A # 88 - 45, La América, Medellín</v>
       </c>
       <c r="G38" t="str">
-        <v>8554832457</v>
+        <v>1715617599</v>
       </c>
       <c r="H38" t="str">
-        <v>Banco AV Villas</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I38" t="str">
-        <v>17/09/2023</v>
+        <v>01/11/2018</v>
       </c>
       <c r="J38" t="str">
         <v>mosorio</v>
@@ -1639,22 +1639,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D39" t="str">
-        <v>848.904.018-9</v>
+        <v>868.438.617-4</v>
       </c>
       <c r="E39" t="str">
-        <v>604 712 68 96</v>
+        <v>604 434 29 32</v>
       </c>
       <c r="F39" t="str">
-        <v>Diagonal 42 # 65 - 44, San Javier, Medellín</v>
+        <v>Transversal 30A # 63 - 59, Rionegro, Medellín</v>
       </c>
       <c r="G39" t="str">
-        <v>4226028136</v>
+        <v>7341135546</v>
       </c>
       <c r="H39" t="str">
-        <v>BBVA Colombia</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I39" t="str">
-        <v>20/03/2017</v>
+        <v>12/03/2019</v>
       </c>
       <c r="J39" t="str">
         <v>mosorio</v>
@@ -1671,22 +1671,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D40" t="str">
-        <v>855.970.931-5</v>
+        <v>891.524.435-2</v>
       </c>
       <c r="E40" t="str">
-        <v>604 350 59 62</v>
+        <v>604 700 77 18</v>
       </c>
       <c r="F40" t="str">
-        <v>Avenida 84 # 13 - 37, La Estrella, Medellín</v>
+        <v>Transversal 39 # 5 - 58, La América, Medellín</v>
       </c>
       <c r="G40" t="str">
-        <v>2157312216</v>
+        <v>3887637394</v>
       </c>
       <c r="H40" t="str">
-        <v>Banco AV Villas</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I40" t="str">
-        <v>28/04/2024</v>
+        <v>05/04/2024</v>
       </c>
       <c r="J40" t="str">
         <v>mosorio</v>
@@ -1703,25 +1703,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D41" t="str">
-        <v>883.339.008-9</v>
+        <v>821.632.325-9</v>
       </c>
       <c r="E41" t="str">
-        <v>604 672 54 40</v>
+        <v>604 855 59 68</v>
       </c>
       <c r="F41" t="str">
-        <v>Transversal 36 # 61 - 36, Rionegro, Medellín</v>
+        <v>Diagonal 16 # 53 - 65, El Poblado, Medellín</v>
       </c>
       <c r="G41" t="str">
-        <v>8654678747</v>
+        <v>8884755674</v>
       </c>
       <c r="H41" t="str">
-        <v>Itaú Colombia</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I41" t="str">
-        <v>26/02/2017</v>
+        <v>03/09/2018</v>
       </c>
       <c r="J41" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="42">
@@ -1735,22 +1735,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D42" t="str">
-        <v>896.599.405-1</v>
+        <v>890.800.681-8</v>
       </c>
       <c r="E42" t="str">
-        <v>604 235 23 12</v>
+        <v>604 645 12 51</v>
       </c>
       <c r="F42" t="str">
-        <v>Calle 16 # 43 - 38, Sabaneta, Medellín</v>
+        <v>Avenida 49A # 45 - 55, Copacabana, Medellín</v>
       </c>
       <c r="G42" t="str">
-        <v>8649590283</v>
+        <v>3295788536</v>
       </c>
       <c r="H42" t="str">
-        <v>Banco AV Villas</v>
+        <v>Banco de Bogotá</v>
       </c>
       <c r="I42" t="str">
-        <v>20/04/2020</v>
+        <v>26/05/2023</v>
       </c>
       <c r="J42" t="str">
         <v>mosorio</v>
@@ -1767,25 +1767,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D43" t="str">
-        <v>837.256.874-0</v>
+        <v>863.644.891-4</v>
       </c>
       <c r="E43" t="str">
-        <v>604 406 83 90</v>
+        <v>604 730 51 28</v>
       </c>
       <c r="F43" t="str">
-        <v>Calle 5 # 81 - 69, Caldas, Medellín</v>
+        <v>Avenida 71 # 32 - 99, El Poblado, Medellín</v>
       </c>
       <c r="G43" t="str">
-        <v>6653092452</v>
+        <v>9560271688</v>
       </c>
       <c r="H43" t="str">
-        <v>Itaú Colombia</v>
+        <v>Banco Agrario de Colombia</v>
       </c>
       <c r="I43" t="str">
-        <v>22/12/2021</v>
+        <v>22/08/2023</v>
       </c>
       <c r="J43" t="str">
-        <v>mosorio</v>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -1799,25 +1799,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D44" t="str">
-        <v>830.504.907-1</v>
+        <v>810.751.516-9</v>
       </c>
       <c r="E44" t="str">
-        <v>604 808 32 25</v>
+        <v>604 326 89 64</v>
       </c>
       <c r="F44" t="str">
-        <v>Diagonal 87 # 4 - 37, Girardota, Medellín</v>
+        <v>Avenida 23A # 6 - 42, Belén, Medellín</v>
       </c>
       <c r="G44" t="str">
-        <v>7525258829</v>
+        <v>9904797384</v>
       </c>
       <c r="H44" t="str">
-        <v>BBVA Colombia</v>
+        <v>Banco de Bogotá</v>
       </c>
       <c r="I44" t="str">
-        <v>23/02/2022</v>
+        <v>06/11/2019</v>
       </c>
       <c r="J44" t="str">
-        <v>mosorio</v>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -1831,22 +1831,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D45" t="str">
-        <v>823.901.254-6</v>
+        <v>810.043.128-7</v>
       </c>
       <c r="E45" t="str">
-        <v>604 351 53 45</v>
+        <v>604 242 16 12</v>
       </c>
       <c r="F45" t="str">
-        <v>Transversal 34 # 11 - 35, Copacabana, Medellín</v>
+        <v>Diagonal 52 # 84 - 11, Guayabal, Medellín</v>
       </c>
       <c r="G45" t="str">
-        <v>3289078526</v>
+        <v>3328847865</v>
       </c>
       <c r="H45" t="str">
-        <v>Davivienda</v>
+        <v>Scotiabank Colpatria</v>
       </c>
       <c r="I45" t="str">
-        <v>13/08/2016</v>
+        <v>06/10/2018</v>
       </c>
       <c r="J45" t="str">
         <v>mosorio</v>
@@ -1863,22 +1863,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D46" t="str">
-        <v>818.472.449-5</v>
+        <v>869.005.382-4</v>
       </c>
       <c r="E46" t="str">
-        <v>604 628 52 47</v>
+        <v>604 516 76 17</v>
       </c>
       <c r="F46" t="str">
-        <v>Diagonal 71 # 81 - 91, Belén, Medellín</v>
+        <v>Calle 78A # 86 - 46, La Estrella, Medellín</v>
       </c>
       <c r="G46" t="str">
-        <v>9846860656</v>
+        <v>3628631733</v>
       </c>
       <c r="H46" t="str">
-        <v>Banco de Bogotá</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I46" t="str">
-        <v>10/05/2019</v>
+        <v>26/06/2016</v>
       </c>
       <c r="J46" t="str">
         <v>mosorio</v>
@@ -1895,22 +1895,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D47" t="str">
-        <v>836.438.587-5</v>
+        <v>832.487.298-6</v>
       </c>
       <c r="E47" t="str">
-        <v>604 824 60 72</v>
+        <v>604 871 26 11</v>
       </c>
       <c r="F47" t="str">
-        <v>Calle 86 # 3 - 17, Sabaneta, Medellín</v>
+        <v>Calle 88 # 88 - 52, Belén, Medellín</v>
       </c>
       <c r="G47" t="str">
-        <v>4903325967</v>
+        <v>4241143111</v>
       </c>
       <c r="H47" t="str">
-        <v>Banco AV Villas</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I47" t="str">
-        <v>23/08/2019</v>
+        <v>10/11/2017</v>
       </c>
       <c r="J47" t="str">
         <v>mosorio</v>
@@ -1927,7 +1927,7 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D48" t="str">
-        <v>829.509.697-7</v>
+        <v>844.603.400-3</v>
       </c>
       <c r="E48" t="str">
         <v>310 486 22 07</v>
@@ -1959,25 +1959,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D49" t="str">
-        <v>802.502.892-7</v>
+        <v>876.863.875-9</v>
       </c>
       <c r="E49" t="str">
-        <v>604 378 64 96</v>
+        <v>604 463 87 26</v>
       </c>
       <c r="F49" t="str">
-        <v>Calle 34 # 48 - 48, Laureles, Medellín</v>
+        <v>Carrera 71 # 9 - 70, Sabaneta, Medellín</v>
       </c>
       <c r="G49" t="str">
-        <v>1658526075</v>
+        <v>8302446652</v>
       </c>
       <c r="H49" t="str">
-        <v>Banco Popular</v>
+        <v>Scotiabank Colpatria</v>
       </c>
       <c r="I49" t="str">
-        <v>01/11/2017</v>
+        <v>18/06/2023</v>
       </c>
       <c r="J49" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="50">
@@ -1991,25 +1991,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D50" t="str">
-        <v>826.036.500-3</v>
+        <v>867.538.145-5</v>
       </c>
       <c r="E50" t="str">
-        <v>604 544 37 30</v>
+        <v>604 855 59 15</v>
       </c>
       <c r="F50" t="str">
-        <v>Diagonal 3 # 16 - 26, La Estrella, Medellín</v>
+        <v>Calle 38 # 40 - 53, Girardota, Medellín</v>
       </c>
       <c r="G50" t="str">
-        <v>1408412140</v>
+        <v>4722271251</v>
       </c>
       <c r="H50" t="str">
-        <v>BBVA Colombia</v>
+        <v>Banco Agrario de Colombia</v>
       </c>
       <c r="I50" t="str">
-        <v>20/09/2021</v>
+        <v>26/07/2019</v>
       </c>
       <c r="J50" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="51">
@@ -2023,22 +2023,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D51" t="str">
-        <v>893.371.353-6</v>
+        <v>889.339.969-3</v>
       </c>
       <c r="E51" t="str">
-        <v>604 513 91 53</v>
+        <v>604 383 52 71</v>
       </c>
       <c r="F51" t="str">
-        <v>Carrera 78 # 43 - 69, El Poblado, Medellín</v>
+        <v>Transversal 78 # 17 - 14, Laureles, Medellín</v>
       </c>
       <c r="G51" t="str">
-        <v>1622570519</v>
+        <v>9389650273</v>
       </c>
       <c r="H51" t="str">
-        <v>Banco AV Villas</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I51" t="str">
-        <v>19/03/2024</v>
+        <v>08/07/2024</v>
       </c>
       <c r="J51" t="str">
         <v>mosorio</v>
@@ -2055,25 +2055,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D52" t="str">
-        <v>834.500.685-6</v>
+        <v>889.554.807-1</v>
       </c>
       <c r="E52" t="str">
-        <v>604 891 48 32</v>
+        <v>604 739 61 68</v>
       </c>
       <c r="F52" t="str">
-        <v>Avenida 78 # 27 - 58, Copacabana, Medellín</v>
+        <v>Avenida 65 # 68 - 39, Envigado, Medellín</v>
       </c>
       <c r="G52" t="str">
-        <v>4909307035</v>
+        <v>5433706704</v>
       </c>
       <c r="H52" t="str">
         <v>Banco AV Villas</v>
       </c>
       <c r="I52" t="str">
-        <v>22/11/2019</v>
+        <v>04/01/2020</v>
       </c>
       <c r="J52" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="53">
@@ -2087,22 +2087,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D53" t="str">
-        <v>839.725.637-7</v>
+        <v>850.512.410-8</v>
       </c>
       <c r="E53" t="str">
-        <v>604 463 21 10</v>
+        <v>604 862 68 96</v>
       </c>
       <c r="F53" t="str">
-        <v>Carrera 63 # 12 - 85, Girardota, Medellín</v>
+        <v>Transversal 31 # 90 - 24, Aranjuez, Medellín</v>
       </c>
       <c r="G53" t="str">
-        <v>7952564249</v>
+        <v>1841894440</v>
       </c>
       <c r="H53" t="str">
-        <v>Banco Popular</v>
+        <v>Davivienda</v>
       </c>
       <c r="I53" t="str">
-        <v>14/02/2024</v>
+        <v>05/03/2017</v>
       </c>
       <c r="J53" t="str">
         <v>mosorio</v>
@@ -2119,22 +2119,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D54" t="str">
-        <v>895.967.263-8</v>
+        <v>874.066.610-8</v>
       </c>
       <c r="E54" t="str">
-        <v>604 788 46 17</v>
+        <v>604 861 94 18</v>
       </c>
       <c r="F54" t="str">
-        <v>Calle 11 # 33 - 14, Bello, Medellín</v>
+        <v>Diagonal 31 # 27 - 70, Belén, Medellín</v>
       </c>
       <c r="G54" t="str">
-        <v>6850289239</v>
+        <v>5252839401</v>
       </c>
       <c r="H54" t="str">
-        <v>Banco de Bogotá</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I54" t="str">
-        <v>02/01/2025</v>
+        <v>30/03/2022</v>
       </c>
       <c r="J54" t="str">
         <v>mosorio</v>
@@ -2151,22 +2151,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D55" t="str">
-        <v>801.857.291-0</v>
+        <v>898.611.876-5</v>
       </c>
       <c r="E55" t="str">
-        <v>604 401 71 11</v>
+        <v>604 529 83 83</v>
       </c>
       <c r="F55" t="str">
-        <v>Calle 6 # 76 - 12, Laureles, Medellín</v>
+        <v>Diagonal 49A # 57 - 33, Itagüí, Medellín</v>
       </c>
       <c r="G55" t="str">
-        <v>4629379201</v>
+        <v>5602227566</v>
       </c>
       <c r="H55" t="str">
-        <v>Banco de Occidente</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I55" t="str">
-        <v>09/01/2025</v>
+        <v>04/06/2020</v>
       </c>
       <c r="J55" t="str">
         <v>mosorio</v>
@@ -2183,22 +2183,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D56" t="str">
-        <v>801.215.763-0</v>
+        <v>816.216.592-7</v>
       </c>
       <c r="E56" t="str">
-        <v>604 842 71 83</v>
+        <v>604 543 30 14</v>
       </c>
       <c r="F56" t="str">
-        <v>Avenida 70 # 88 - 87, El Poblado, Medellín</v>
+        <v>Diagonal 88A # 78 - 18, Belén, Medellín</v>
       </c>
       <c r="G56" t="str">
-        <v>3708612165</v>
+        <v>6582102182</v>
       </c>
       <c r="H56" t="str">
-        <v>BBVA Colombia</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I56" t="str">
-        <v>05/04/2023</v>
+        <v>09/12/2023</v>
       </c>
       <c r="J56" t="str">
         <v/>
@@ -2215,22 +2215,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D57" t="str">
-        <v>863.526.546-9</v>
+        <v>857.696.914-2</v>
       </c>
       <c r="E57" t="str">
-        <v>604 880 37 24</v>
+        <v>604 600 64 90</v>
       </c>
       <c r="F57" t="str">
-        <v>Calle 10 # 64 - 53, Robledo, Medellín</v>
+        <v>Diagonal 57A # 2 - 58, Guayabal, Medellín</v>
       </c>
       <c r="G57" t="str">
-        <v>7898800747</v>
+        <v>4815082769</v>
       </c>
       <c r="H57" t="str">
-        <v>Davivienda</v>
+        <v>Scotiabank Colpatria</v>
       </c>
       <c r="I57" t="str">
-        <v>23/02/2019</v>
+        <v>02/11/2021</v>
       </c>
       <c r="J57" t="str">
         <v>mosorio</v>
@@ -2247,22 +2247,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D58" t="str">
-        <v>892.500.398-8</v>
+        <v>849.605.537-0</v>
       </c>
       <c r="E58" t="str">
-        <v>604 587 15 76</v>
+        <v>604 670 33 26</v>
       </c>
       <c r="F58" t="str">
-        <v>Carrera 8 # 32 - 61, Robledo, Medellín</v>
+        <v>Transversal 43A # 96 - 40, Caldas, Medellín</v>
       </c>
       <c r="G58" t="str">
-        <v>1563275328</v>
+        <v>3240036919</v>
       </c>
       <c r="H58" t="str">
-        <v>Davivienda</v>
+        <v>Banco de Occidente</v>
       </c>
       <c r="I58" t="str">
-        <v>08/08/2017</v>
+        <v>07/09/2022</v>
       </c>
       <c r="J58" t="str">
         <v>mosorio</v>
@@ -2279,22 +2279,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D59" t="str">
-        <v>855.896.181-1</v>
+        <v>810.061.543-7</v>
       </c>
       <c r="E59" t="str">
-        <v>604 759 64 43</v>
+        <v>604 489 88 65</v>
       </c>
       <c r="F59" t="str">
-        <v>Avenida 76 # 37 - 16, El Poblado, Medellín</v>
+        <v>Calle 8 # 58 - 74, Girardota, Medellín</v>
       </c>
       <c r="G59" t="str">
-        <v>9777062303</v>
+        <v>1553933831</v>
       </c>
       <c r="H59" t="str">
         <v>Scotiabank Colpatria</v>
       </c>
       <c r="I59" t="str">
-        <v>18/05/2019</v>
+        <v>19/05/2019</v>
       </c>
       <c r="J59" t="str">
         <v>mosorio</v>
@@ -2311,22 +2311,22 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D60" t="str">
-        <v>834.225.612-1</v>
+        <v>820.680.469-1</v>
       </c>
       <c r="E60" t="str">
-        <v>604 731 35 85</v>
+        <v>604 393 87 71</v>
       </c>
       <c r="F60" t="str">
-        <v>Avenida 21 # 12 - 68, Sabaneta, Medellín</v>
+        <v>Transversal 16 # 54 - 49, Bello, Medellín</v>
       </c>
       <c r="G60" t="str">
-        <v>4222560157</v>
+        <v>6705419236</v>
       </c>
       <c r="H60" t="str">
-        <v>BBVA Colombia</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I60" t="str">
-        <v>05/04/2023</v>
+        <v>19/11/2022</v>
       </c>
       <c r="J60" t="str">
         <v>mosorio</v>
@@ -2343,25 +2343,25 @@
         <v>PROVEEDOR</v>
       </c>
       <c r="D61" t="str">
-        <v>803.797.028-9</v>
+        <v>886.586.309-1</v>
       </c>
       <c r="E61" t="str">
-        <v>604 241 70 24</v>
+        <v>604 768 28 11</v>
       </c>
       <c r="F61" t="str">
-        <v>Transversal 25 # 59 - 66, Bello, Medellín</v>
+        <v>Transversal 50 # 91 - 81, Rionegro, Medellín</v>
       </c>
       <c r="G61" t="str">
-        <v>2923832717</v>
+        <v>9649365890</v>
       </c>
       <c r="H61" t="str">
-        <v>Banco AV Villas</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I61" t="str">
-        <v>26/12/2024</v>
+        <v>01/07/2019</v>
       </c>
       <c r="J61" t="str">
-        <v/>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="62">
@@ -2375,25 +2375,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D62" t="str">
-        <v>937.881.376-2</v>
+        <v>974.447.511-5</v>
       </c>
       <c r="E62" t="str">
-        <v>604 541 71 67</v>
+        <v>327 452 20 60</v>
       </c>
       <c r="F62" t="str">
-        <v>Calle 20 # 59 - 95, Guayabal, Medellín</v>
+        <v>Diagonal 11 # 4 - 45, Bello, Medellín</v>
       </c>
       <c r="G62" t="str">
-        <v>2605511856</v>
+        <v>1815230258</v>
       </c>
       <c r="H62" t="str">
-        <v>Banco de Bogotá</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I62" t="str">
-        <v>11/05/2024</v>
+        <v>07/10/2022</v>
       </c>
       <c r="J62" t="str">
-        <v>dcastro</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="63">
@@ -2407,25 +2407,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D63" t="str">
-        <v>925.888.643-2</v>
+        <v>983.853.723-3</v>
       </c>
       <c r="E63" t="str">
-        <v>604 463 47 94</v>
+        <v>604 542 75 68</v>
       </c>
       <c r="F63" t="str">
-        <v>Avenida 50 # 89 - 57, Copacabana, Medellín</v>
+        <v>Avenida 61 # 32 - 68, Bello, Medellín</v>
       </c>
       <c r="G63" t="str">
-        <v>6809769989</v>
+        <v>7402971211</v>
       </c>
       <c r="H63" t="str">
-        <v>Scotiabank Colpatria</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I63" t="str">
-        <v>10/12/2022</v>
+        <v>09/11/2019</v>
       </c>
       <c r="J63" t="str">
-        <v>dcastro</v>
+        <v>lramos</v>
       </c>
     </row>
     <row r="64">
@@ -2439,25 +2439,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D64" t="str">
-        <v>963.413.934-0</v>
+        <v>917.930.919-1</v>
       </c>
       <c r="E64" t="str">
-        <v>604 539 44 69</v>
+        <v>305 610 88 86</v>
       </c>
       <c r="F64" t="str">
-        <v>Transversal 6 # 97 - 39, Castilla, Medellín</v>
+        <v>Carrera 13 # 81 - 26, Laureles, Medellín</v>
       </c>
       <c r="G64" t="str">
-        <v>6824762411</v>
+        <v>6828677859</v>
       </c>
       <c r="H64" t="str">
-        <v>Banco de Occidente</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I64" t="str">
-        <v>21/01/2022</v>
+        <v>05/10/2023</v>
       </c>
       <c r="J64" t="str">
-        <v>dcastro</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="65">
@@ -2471,22 +2471,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D65" t="str">
-        <v>970.000.737-9</v>
+        <v>949.752.429-5</v>
       </c>
       <c r="E65" t="str">
-        <v>307 372 46 38</v>
+        <v>604 487 42 92</v>
       </c>
       <c r="F65" t="str">
-        <v>Carrera 76 # 19 - 32, El Poblado, Medellín</v>
+        <v>Diagonal 29 # 78 - 65, Copacabana, Medellín</v>
       </c>
       <c r="G65" t="str">
-        <v>8778292148</v>
+        <v>6177393709</v>
       </c>
       <c r="H65" t="str">
-        <v>Itaú Colombia</v>
+        <v>Banco Agrario de Colombia</v>
       </c>
       <c r="I65" t="str">
-        <v>09/12/2022</v>
+        <v>28/06/2017</v>
       </c>
       <c r="J65" t="str">
         <v>lramos</v>
@@ -2503,25 +2503,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D66" t="str">
-        <v>935.489.623-1</v>
+        <v>903.330.632-6</v>
       </c>
       <c r="E66" t="str">
-        <v>604 732 11 33</v>
+        <v>604 313 66 48</v>
       </c>
       <c r="F66" t="str">
-        <v>Avenida 59 # 31 - 36, Sabaneta, Medellín</v>
+        <v>Carrera 33 # 61 - 42, La Estrella, Medellín</v>
       </c>
       <c r="G66" t="str">
-        <v>4294175456</v>
+        <v>5438369003</v>
       </c>
       <c r="H66" t="str">
         <v>Banco de Bogotá</v>
       </c>
       <c r="I66" t="str">
-        <v>14/10/2017</v>
+        <v>07/08/2023</v>
       </c>
       <c r="J66" t="str">
-        <v>lramos</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="67">
@@ -2535,25 +2535,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D67" t="str">
-        <v>945.183.420-3</v>
+        <v>915.758.079-4</v>
       </c>
       <c r="E67" t="str">
-        <v>604 702 22 62</v>
+        <v>604 684 82 69</v>
       </c>
       <c r="F67" t="str">
-        <v>Diagonal 97 # 52 - 74, Girardota, Medellín</v>
+        <v>Avenida 59 # 23 - 62, Aranjuez, Medellín</v>
       </c>
       <c r="G67" t="str">
-        <v>4510936554</v>
+        <v>6370963438</v>
       </c>
       <c r="H67" t="str">
-        <v>Banco AV Villas</v>
+        <v>Banco de Bogotá</v>
       </c>
       <c r="I67" t="str">
-        <v>23/08/2022</v>
+        <v>14/06/2018</v>
       </c>
       <c r="J67" t="str">
-        <v>kalzate</v>
+        <v>dcastro</v>
       </c>
     </row>
     <row r="68">
@@ -2567,22 +2567,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D68" t="str">
-        <v>987.009.682-5</v>
+        <v>987.253.740-9</v>
       </c>
       <c r="E68" t="str">
-        <v>316 488 51 63</v>
+        <v>303 863 72 52</v>
       </c>
       <c r="F68" t="str">
-        <v>Avenida 3 # 2 - 37, Caldas, Medellín</v>
+        <v>Avenida 37 # 6 - 31, Envigado, Medellín</v>
       </c>
       <c r="G68" t="str">
-        <v>6393498145</v>
+        <v>5458875545</v>
       </c>
       <c r="H68" t="str">
-        <v>Banco de Bogotá</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I68" t="str">
-        <v>11/08/2017</v>
+        <v>14/08/2021</v>
       </c>
       <c r="J68" t="str">
         <v>lramos</v>
@@ -2599,22 +2599,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D69" t="str">
-        <v>958.573.735-9</v>
+        <v>929.001.545-7</v>
       </c>
       <c r="E69" t="str">
-        <v>324 304 30 54</v>
+        <v>302 647 25 12</v>
       </c>
       <c r="F69" t="str">
-        <v>Carrera 38 # 65 - 98, Castilla, Medellín</v>
+        <v>Transversal 18 # 47 - 47, Copacabana, Medellín</v>
       </c>
       <c r="G69" t="str">
-        <v>5419241195</v>
+        <v>7325122768</v>
       </c>
       <c r="H69" t="str">
-        <v>Banco AV Villas</v>
+        <v>Banco Agrario de Colombia</v>
       </c>
       <c r="I69" t="str">
-        <v>31/05/2022</v>
+        <v>21/11/2017</v>
       </c>
       <c r="J69" t="str">
         <v>kalzate</v>
@@ -2631,25 +2631,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D70" t="str">
-        <v>917.976.111-4</v>
+        <v>982.324.828-5</v>
       </c>
       <c r="E70" t="str">
-        <v>321 748 10 12</v>
+        <v>303 440 42 90</v>
       </c>
       <c r="F70" t="str">
-        <v>Carrera 48 # 17 - 59, Manrique, Medellín</v>
+        <v>Transversal 69A # 87 - 37, El Poblado, Medellín</v>
       </c>
       <c r="G70" t="str">
-        <v>8696933434</v>
+        <v>1391468933</v>
       </c>
       <c r="H70" t="str">
-        <v>Banco de Bogotá</v>
+        <v>Banco AV Villas</v>
       </c>
       <c r="I70" t="str">
-        <v>26/11/2022</v>
+        <v>07/03/2023</v>
       </c>
       <c r="J70" t="str">
-        <v>lramos</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="71">
@@ -2663,22 +2663,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D71" t="str">
-        <v>977.747.652-3</v>
+        <v>937.652.252-6</v>
       </c>
       <c r="E71" t="str">
-        <v>300 689 92 60</v>
+        <v>604 403 42 92</v>
       </c>
       <c r="F71" t="str">
-        <v>Transversal 60 # 28 - 97, Caldas, Medellín</v>
+        <v>Avenida 80 # 4 - 33, Guayabal, Medellín</v>
       </c>
       <c r="G71" t="str">
-        <v>3258748593</v>
+        <v>6334998836</v>
       </c>
       <c r="H71" t="str">
-        <v>Bancolombia</v>
+        <v>Banco AV Villas</v>
       </c>
       <c r="I71" t="str">
-        <v>17/10/2019</v>
+        <v>21/02/2022</v>
       </c>
       <c r="J71" t="str">
         <v>lramos</v>
@@ -2695,22 +2695,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D72" t="str">
-        <v>968.614.370-8</v>
+        <v>909.799.814-5</v>
       </c>
       <c r="E72" t="str">
-        <v>327 749 71 93</v>
+        <v>604 378 64 96</v>
       </c>
       <c r="F72" t="str">
-        <v>Avenida 44 # 45 - 54, Rionegro, Medellín</v>
+        <v>Calle 34 # 48 - 48, Laureles, Medellín</v>
       </c>
       <c r="G72" t="str">
-        <v>5614968774</v>
+        <v>1658526075</v>
       </c>
       <c r="H72" t="str">
-        <v>Scotiabank Colpatria</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I72" t="str">
-        <v>27/05/2022</v>
+        <v>24/05/2018</v>
       </c>
       <c r="J72" t="str">
         <v>kalzate</v>
@@ -2727,25 +2727,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D73" t="str">
-        <v>938.643.148-3</v>
+        <v>926.036.500-6</v>
       </c>
       <c r="E73" t="str">
-        <v>317 510 29 56</v>
+        <v>604 415 30 67</v>
       </c>
       <c r="F73" t="str">
-        <v>Transversal 32 # 25 - 47, Envigado, Medellín</v>
+        <v>Calle 85A # 19 - 86, Laureles, Medellín</v>
       </c>
       <c r="G73" t="str">
-        <v>8100117595</v>
+        <v>4188565123</v>
       </c>
       <c r="H73" t="str">
-        <v>Banco Agrario de Colombia</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I73" t="str">
-        <v>21/02/2022</v>
+        <v>02/11/2024</v>
       </c>
       <c r="J73" t="str">
-        <v>lramos</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="74">
@@ -2759,22 +2759,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D74" t="str">
-        <v>929.084.778-1</v>
+        <v>944.927.052-7</v>
       </c>
       <c r="E74" t="str">
-        <v>604 564 91 82</v>
+        <v>312 753 50 48</v>
       </c>
       <c r="F74" t="str">
-        <v>Transversal 86A # 21 - 97, Aranjuez, Medellín</v>
+        <v>Diagonal 3A # 58 - 94, La Estrella, Medellín</v>
       </c>
       <c r="G74" t="str">
-        <v>7149038995</v>
+        <v>9148586003</v>
       </c>
       <c r="H74" t="str">
-        <v>Banco Popular</v>
+        <v>Banco Agrario de Colombia</v>
       </c>
       <c r="I74" t="str">
-        <v>13/08/2023</v>
+        <v>07/07/2020</v>
       </c>
       <c r="J74" t="str">
         <v>lramos</v>
@@ -2791,25 +2791,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D75" t="str">
-        <v>942.806.052-0</v>
+        <v>983.859.919-7</v>
       </c>
       <c r="E75" t="str">
-        <v>314 427 30 53</v>
+        <v>322 574 78 47</v>
       </c>
       <c r="F75" t="str">
-        <v>Carrera 44 # 77 - 31, Manrique, Medellín</v>
+        <v>Avenida 57 # 40 - 64, Bello, Medellín</v>
       </c>
       <c r="G75" t="str">
-        <v>3601453503</v>
+        <v>4213852820</v>
       </c>
       <c r="H75" t="str">
-        <v>Bancolombia</v>
+        <v>Banco de Bogotá</v>
       </c>
       <c r="I75" t="str">
-        <v>01/11/2023</v>
+        <v>10/03/2022</v>
       </c>
       <c r="J75" t="str">
-        <v>lramos</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="76">
@@ -2823,25 +2823,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D76" t="str">
-        <v>975.134.003-5</v>
+        <v>912.848.078-2</v>
       </c>
       <c r="E76" t="str">
-        <v>318 704 60 49</v>
+        <v>327 863 92 67</v>
       </c>
       <c r="F76" t="str">
-        <v>Transversal 82 # 15 - 99, Laureles, Medellín</v>
+        <v>Avenida 33 # 84 - 46, Laureles, Medellín</v>
       </c>
       <c r="G76" t="str">
-        <v>7360404549</v>
+        <v>2193313658</v>
       </c>
       <c r="H76" t="str">
-        <v>Scotiabank Colpatria</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I76" t="str">
-        <v>25/06/2017</v>
+        <v>18/06/2017</v>
       </c>
       <c r="J76" t="str">
-        <v>kalzate</v>
+        <v>dcastro</v>
       </c>
     </row>
     <row r="77">
@@ -2855,25 +2855,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D77" t="str">
-        <v>937.788.123-9</v>
+        <v>961.272.995-6</v>
       </c>
       <c r="E77" t="str">
-        <v>302 496 41 12</v>
+        <v>322 897 23 10</v>
       </c>
       <c r="F77" t="str">
-        <v>Transversal 1 # 55 - 54, Manrique, Medellín</v>
+        <v>Carrera 68A # 15 - 14, Sabaneta, Medellín</v>
       </c>
       <c r="G77" t="str">
-        <v>1986607761</v>
+        <v>7129363570</v>
       </c>
       <c r="H77" t="str">
-        <v>Banco Popular</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I77" t="str">
-        <v>17/09/2022</v>
+        <v>04/10/2021</v>
       </c>
       <c r="J77" t="str">
-        <v>kalzate</v>
+        <v>lramos</v>
       </c>
     </row>
     <row r="78">
@@ -2887,25 +2887,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D78" t="str">
-        <v>934.283.043-2</v>
+        <v>946.058.010-9</v>
       </c>
       <c r="E78" t="str">
-        <v>604 477 30 15</v>
+        <v>300 842 71 83</v>
       </c>
       <c r="F78" t="str">
-        <v>Calle 60A # 87 - 54, San Javier, Medellín</v>
+        <v>Avenida 70 # 88 - 87, El Poblado, Medellín</v>
       </c>
       <c r="G78" t="str">
-        <v>8221903263</v>
+        <v>3708612165</v>
       </c>
       <c r="H78" t="str">
-        <v>Davivienda</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I78" t="str">
-        <v>15/01/2024</v>
+        <v>21/05/2023</v>
       </c>
       <c r="J78" t="str">
-        <v>lramos</v>
+        <v>dcastro</v>
       </c>
     </row>
     <row r="79">
@@ -2919,22 +2919,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D79" t="str">
-        <v>938.474.215-3</v>
+        <v>963.526.546-1</v>
       </c>
       <c r="E79" t="str">
-        <v>315 541 23 11</v>
+        <v>301 299 18 96</v>
       </c>
       <c r="F79" t="str">
-        <v>Transversal 65A # 87 - 91, Robledo, Medellín</v>
+        <v>Diagonal 47 # 69 - 89, Copacabana, Medellín</v>
       </c>
       <c r="G79" t="str">
-        <v>4859215019</v>
+        <v>2384848431</v>
       </c>
       <c r="H79" t="str">
-        <v>Itaú Colombia</v>
+        <v>Banco Agrario de Colombia</v>
       </c>
       <c r="I79" t="str">
-        <v>18/08/2024</v>
+        <v>24/06/2021</v>
       </c>
       <c r="J79" t="str">
         <v>lramos</v>
@@ -2951,22 +2951,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D80" t="str">
-        <v>967.051.866-8</v>
+        <v>973.871.021-1</v>
       </c>
       <c r="E80" t="str">
-        <v>307 336 85 15</v>
+        <v>604 253 75 38</v>
       </c>
       <c r="F80" t="str">
-        <v>Carrera 10 # 82 - 71, Manrique, Medellín</v>
+        <v>Transversal 42A # 51 - 85, Guayabal, Medellín</v>
       </c>
       <c r="G80" t="str">
-        <v>5260862391</v>
+        <v>2639458815</v>
       </c>
       <c r="H80" t="str">
-        <v>Davivienda</v>
+        <v>Scotiabank Colpatria</v>
       </c>
       <c r="I80" t="str">
-        <v>12/02/2023</v>
+        <v>24/11/2021</v>
       </c>
       <c r="J80" t="str">
         <v>dcastro</v>
@@ -2983,25 +2983,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D81" t="str">
-        <v>909.749.820-6</v>
+        <v>990.380.600-0</v>
       </c>
       <c r="E81" t="str">
-        <v>308 550 78 82</v>
+        <v>323 247 12 95</v>
       </c>
       <c r="F81" t="str">
-        <v>Avenida 34 # 46 - 87, Sabaneta, Medellín</v>
+        <v>Diagonal 39 # 34 - 59, Sabaneta, Medellín</v>
       </c>
       <c r="G81" t="str">
-        <v>6122071586</v>
+        <v>7352420008</v>
       </c>
       <c r="H81" t="str">
-        <v>Davivienda</v>
+        <v>Banco AV Villas</v>
       </c>
       <c r="I81" t="str">
-        <v>14/02/2020</v>
+        <v>16/09/2018</v>
       </c>
       <c r="J81" t="str">
-        <v>dcastro</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="82">
@@ -3015,25 +3015,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D82" t="str">
-        <v>980.307.508-4</v>
+        <v>912.441.505-8</v>
       </c>
       <c r="E82" t="str">
-        <v>604 221 99 69</v>
+        <v>314 295 80 43</v>
       </c>
       <c r="F82" t="str">
-        <v>Calle 28 # 60 - 19, Sabaneta, Medellín</v>
+        <v>Diagonal 21A # 6 - 70, Guayabal, Medellín</v>
       </c>
       <c r="G82" t="str">
-        <v>6737440645</v>
+        <v>6325538763</v>
       </c>
       <c r="H82" t="str">
-        <v>BBVA Colombia</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I82" t="str">
-        <v>22/09/2020</v>
+        <v>30/01/2022</v>
       </c>
       <c r="J82" t="str">
-        <v>lramos</v>
+        <v>dcastro</v>
       </c>
     </row>
     <row r="83">
@@ -3047,22 +3047,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D83" t="str">
-        <v>996.531.603-3</v>
+        <v>919.163.088-0</v>
       </c>
       <c r="E83" t="str">
-        <v>312 587 22 89</v>
+        <v>328 895 71 43</v>
       </c>
       <c r="F83" t="str">
-        <v>Transversal 79 # 94 - 95, Castilla, Medellín</v>
+        <v>Calle 48 # 64 - 13, Envigado, Medellín</v>
       </c>
       <c r="G83" t="str">
-        <v>8287063299</v>
+        <v>8634730279</v>
       </c>
       <c r="H83" t="str">
-        <v>Banco de Bogotá</v>
+        <v>Davivienda</v>
       </c>
       <c r="I83" t="str">
-        <v>11/03/2023</v>
+        <v>21/02/2018</v>
       </c>
       <c r="J83" t="str">
         <v>dcastro</v>
@@ -3079,25 +3079,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D84" t="str">
-        <v>995.523.674-9</v>
+        <v>964.657.204-3</v>
       </c>
       <c r="E84" t="str">
-        <v>604 804 70 29</v>
+        <v>604 840 69 32</v>
       </c>
       <c r="F84" t="str">
-        <v>Diagonal 66 # 81 - 93, Copacabana, Medellín</v>
+        <v>Carrera 37 # 93 - 91, Buenos Aires, Medellín</v>
       </c>
       <c r="G84" t="str">
-        <v>3296848016</v>
+        <v>7901921385</v>
       </c>
       <c r="H84" t="str">
-        <v>Banco Popular</v>
+        <v>Scotiabank Colpatria</v>
       </c>
       <c r="I84" t="str">
-        <v>02/07/2024</v>
+        <v>12/05/2022</v>
       </c>
       <c r="J84" t="str">
-        <v>lramos</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="85">
@@ -3111,25 +3111,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D85" t="str">
-        <v>964.963.793-1</v>
+        <v>996.699.893-4</v>
       </c>
       <c r="E85" t="str">
-        <v>318 462 56 96</v>
+        <v>324 645 16 53</v>
       </c>
       <c r="F85" t="str">
-        <v>Transversal 43 # 1 - 73, Belén, Medellín</v>
+        <v>Carrera 65 # 6 - 40, Rionegro, Medellín</v>
       </c>
       <c r="G85" t="str">
-        <v>5812291592</v>
+        <v>3599565225</v>
       </c>
       <c r="H85" t="str">
         <v>Banco AV Villas</v>
       </c>
       <c r="I85" t="str">
-        <v>12/05/2024</v>
+        <v>05/05/2018</v>
       </c>
       <c r="J85" t="str">
-        <v>kalzate</v>
+        <v>dcastro</v>
       </c>
     </row>
     <row r="86">
@@ -3143,25 +3143,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D86" t="str">
-        <v>923.441.348-8</v>
+        <v>962.327.434-8</v>
       </c>
       <c r="E86" t="str">
-        <v>604 803 57 43</v>
+        <v>604 692 77 16</v>
       </c>
       <c r="F86" t="str">
-        <v>Transversal 42 # 6 - 22, La América, Medellín</v>
+        <v>Diagonal 25 # 32 - 35, Copacabana, Medellín</v>
       </c>
       <c r="G86" t="str">
-        <v>8780037279</v>
+        <v>9265194042</v>
       </c>
       <c r="H86" t="str">
-        <v>Scotiabank Colpatria</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I86" t="str">
-        <v>28/10/2023</v>
+        <v>27/04/2023</v>
       </c>
       <c r="J86" t="str">
-        <v>lramos</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="87">
@@ -3175,25 +3175,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D87" t="str">
-        <v>993.409.013-6</v>
+        <v>988.036.292-4</v>
       </c>
       <c r="E87" t="str">
-        <v>604 650 59 99</v>
+        <v>320 446 19 78</v>
       </c>
       <c r="F87" t="str">
-        <v>Avenida 75A # 23 - 57, Sabaneta, Medellín</v>
+        <v>Calle 26 # 59 - 84, Sabaneta, Medellín</v>
       </c>
       <c r="G87" t="str">
-        <v>8317229967</v>
+        <v>3412988844</v>
       </c>
       <c r="H87" t="str">
-        <v>Banco de Occidente</v>
+        <v>Banco de Bogotá</v>
       </c>
       <c r="I87" t="str">
-        <v>27/04/2017</v>
+        <v>04/05/2022</v>
       </c>
       <c r="J87" t="str">
-        <v>dcastro</v>
+        <v>lramos</v>
       </c>
     </row>
     <row r="88">
@@ -3207,22 +3207,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D88" t="str">
-        <v>976.536.851-3</v>
+        <v>909.641.731-3</v>
       </c>
       <c r="E88" t="str">
-        <v>604 548 99 53</v>
+        <v>604 515 10 74</v>
       </c>
       <c r="F88" t="str">
-        <v>Carrera 17A # 15 - 82, Aranjuez, Medellín</v>
+        <v>Calle 57 # 98 - 70, Buenos Aires, Medellín</v>
       </c>
       <c r="G88" t="str">
-        <v>3202171658</v>
+        <v>7928706114</v>
       </c>
       <c r="H88" t="str">
         <v>Banco de Occidente</v>
       </c>
       <c r="I88" t="str">
-        <v>29/06/2024</v>
+        <v>23/07/2020</v>
       </c>
       <c r="J88" t="str">
         <v>kalzate</v>
@@ -3239,22 +3239,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D89" t="str">
-        <v>937.463.437-0</v>
+        <v>969.567.674-3</v>
       </c>
       <c r="E89" t="str">
-        <v>604 362 34 70</v>
+        <v>326 522 69 47</v>
       </c>
       <c r="F89" t="str">
-        <v>Avenida 95 # 57 - 23, Buenos Aires, Medellín</v>
+        <v>Transversal 58 # 3 - 44, El Poblado, Medellín</v>
       </c>
       <c r="G89" t="str">
-        <v>6157645727</v>
+        <v>3874183376</v>
       </c>
       <c r="H89" t="str">
-        <v>Bancolombia</v>
+        <v>BBVA Colombia</v>
       </c>
       <c r="I89" t="str">
-        <v>08/01/2018</v>
+        <v>06/03/2021</v>
       </c>
       <c r="J89" t="str">
         <v>lramos</v>
@@ -3271,25 +3271,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D90" t="str">
-        <v>993.267.143-4</v>
+        <v>907.454.540-4</v>
       </c>
       <c r="E90" t="str">
-        <v>303 365 52 66</v>
+        <v>604 611 79 75</v>
       </c>
       <c r="F90" t="str">
-        <v>Transversal 51 # 5 - 97, Bello, Medellín</v>
+        <v>Transversal 15A # 49 - 37, Bello, Medellín</v>
       </c>
       <c r="G90" t="str">
-        <v>1308440032</v>
+        <v>4686024209</v>
       </c>
       <c r="H90" t="str">
-        <v>Banco AV Villas</v>
+        <v>Itaú Colombia</v>
       </c>
       <c r="I90" t="str">
-        <v>23/09/2020</v>
+        <v>25/05/2021</v>
       </c>
       <c r="J90" t="str">
-        <v>lramos</v>
+        <v>dcastro</v>
       </c>
     </row>
     <row r="91">
@@ -3303,25 +3303,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D91" t="str">
-        <v>956.860.754-2</v>
+        <v>953.073.554-9</v>
       </c>
       <c r="E91" t="str">
-        <v>321 729 98 31</v>
+        <v>329 321 98 74</v>
       </c>
       <c r="F91" t="str">
-        <v>Avenida 31 # 21 - 54, Manrique, Medellín</v>
+        <v>Calle 77A # 3 - 36, La América, Medellín</v>
       </c>
       <c r="G91" t="str">
-        <v>3125752614</v>
+        <v>5248031935</v>
       </c>
       <c r="H91" t="str">
         <v>Banco Popular</v>
       </c>
       <c r="I91" t="str">
-        <v>13/09/2023</v>
+        <v>18/05/2023</v>
       </c>
       <c r="J91" t="str">
-        <v>kalzate</v>
+        <v>dcastro</v>
       </c>
     </row>
     <row r="92">
@@ -3335,25 +3335,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D92" t="str">
-        <v>988.835.149-7</v>
+        <v>947.138.233-9</v>
       </c>
       <c r="E92" t="str">
-        <v>604 261 59 97</v>
+        <v>604 712 11 80</v>
       </c>
       <c r="F92" t="str">
-        <v>Carrera 86A # 98 - 93, La Estrella, Medellín</v>
+        <v>Avenida 32A # 70 - 92, Castilla, Medellín</v>
       </c>
       <c r="G92" t="str">
-        <v>4402475828</v>
+        <v>5649429592</v>
       </c>
       <c r="H92" t="str">
-        <v>Banco Agrario de Colombia</v>
+        <v>Banco de Bogotá</v>
       </c>
       <c r="I92" t="str">
-        <v>10/01/2024</v>
+        <v>27/10/2024</v>
       </c>
       <c r="J92" t="str">
-        <v>dcastro</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="93">
@@ -3367,22 +3367,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D93" t="str">
-        <v>957.566.266-3</v>
+        <v>922.961.521-3</v>
       </c>
       <c r="E93" t="str">
-        <v>604 338 78 32</v>
+        <v>604 445 11 40</v>
       </c>
       <c r="F93" t="str">
-        <v>Transversal 86 # 28 - 45, Sabaneta, Medellín</v>
+        <v>Calle 68 # 75 - 78, Copacabana, Medellín</v>
       </c>
       <c r="G93" t="str">
-        <v>5199349244</v>
+        <v>7932510369</v>
       </c>
       <c r="H93" t="str">
-        <v>Davivienda</v>
+        <v>Banco de Occidente</v>
       </c>
       <c r="I93" t="str">
-        <v>18/03/2019</v>
+        <v>09/04/2021</v>
       </c>
       <c r="J93" t="str">
         <v>dcastro</v>
@@ -3399,22 +3399,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D94" t="str">
-        <v>929.339.888-4</v>
+        <v>948.950.215-4</v>
       </c>
       <c r="E94" t="str">
-        <v>604 702 87 98</v>
+        <v>315 489 80 70</v>
       </c>
       <c r="F94" t="str">
-        <v>Transversal 20 # 55 - 42, Sabaneta, Medellín</v>
+        <v>Diagonal 38 # 42 - 77, Robledo, Medellín</v>
       </c>
       <c r="G94" t="str">
-        <v>7639702171</v>
+        <v>2568847064</v>
       </c>
       <c r="H94" t="str">
         <v>BBVA Colombia</v>
       </c>
       <c r="I94" t="str">
-        <v>03/03/2024</v>
+        <v>16/07/2024</v>
       </c>
       <c r="J94" t="str">
         <v>lramos</v>
@@ -3431,25 +3431,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D95" t="str">
-        <v>983.176.277-5</v>
+        <v>941.908.866-3</v>
       </c>
       <c r="E95" t="str">
-        <v>604 631 43 31</v>
+        <v>604 811 10 59</v>
       </c>
       <c r="F95" t="str">
-        <v>Carrera 50 # 57 - 61, La América, Medellín</v>
+        <v>Avenida 63A # 29 - 40, Buenos Aires, Medellín</v>
       </c>
       <c r="G95" t="str">
-        <v>6890869747</v>
+        <v>9823846515</v>
       </c>
       <c r="H95" t="str">
-        <v>BBVA Colombia</v>
+        <v>Banco AV Villas</v>
       </c>
       <c r="I95" t="str">
-        <v>30/11/2020</v>
+        <v>02/06/2017</v>
       </c>
       <c r="J95" t="str">
-        <v>kalzate</v>
+        <v>lramos</v>
       </c>
     </row>
     <row r="96">
@@ -3463,25 +3463,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D96" t="str">
-        <v>919.638.740-5</v>
+        <v>996.598.425-7</v>
       </c>
       <c r="E96" t="str">
-        <v>314 703 30 69</v>
+        <v>320 594 71 83</v>
       </c>
       <c r="F96" t="str">
-        <v>Transversal 88A # 11 - 94, Girardota, Medellín</v>
+        <v>Calle 42 # 55 - 48, Sabaneta, Medellín</v>
       </c>
       <c r="G96" t="str">
-        <v>2552438711</v>
+        <v>3532373652</v>
       </c>
       <c r="H96" t="str">
-        <v>Itaú Colombia</v>
+        <v>Banco de Occidente</v>
       </c>
       <c r="I96" t="str">
-        <v>14/02/2017</v>
+        <v>02/10/2024</v>
       </c>
       <c r="J96" t="str">
-        <v>dcastro</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="97">
@@ -3495,22 +3495,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D97" t="str">
-        <v>910.340.030-0</v>
+        <v>923.968.709-6</v>
       </c>
       <c r="E97" t="str">
-        <v>308 826 70 22</v>
+        <v>305 474 10 86</v>
       </c>
       <c r="F97" t="str">
-        <v>Calle 78 # 70 - 85, Castilla, Medellín</v>
+        <v>Carrera 75 # 45 - 86, San Javier, Medellín</v>
       </c>
       <c r="G97" t="str">
-        <v>6767398016</v>
+        <v>6496035924</v>
       </c>
       <c r="H97" t="str">
         <v>Banco AV Villas</v>
       </c>
       <c r="I97" t="str">
-        <v>03/10/2017</v>
+        <v>31/12/2022</v>
       </c>
       <c r="J97" t="str">
         <v>lramos</v>
@@ -3527,25 +3527,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D98" t="str">
-        <v>979.676.950-5</v>
+        <v>998.585.648-3</v>
       </c>
       <c r="E98" t="str">
-        <v>325 666 94 29</v>
+        <v>604 737 36 98</v>
       </c>
       <c r="F98" t="str">
-        <v>Diagonal 85 # 40 - 46, Aranjuez, Medellín</v>
+        <v>Diagonal 5 # 38 - 76, Itagüí, Medellín</v>
       </c>
       <c r="G98" t="str">
-        <v>7701536885</v>
+        <v>3481491633</v>
       </c>
       <c r="H98" t="str">
-        <v>Banco Popular</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I98" t="str">
-        <v>24/05/2018</v>
+        <v>06/06/2021</v>
       </c>
       <c r="J98" t="str">
-        <v>dcastro</v>
+        <v>lramos</v>
       </c>
     </row>
     <row r="99">
@@ -3559,25 +3559,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D99" t="str">
-        <v>920.773.808-8</v>
+        <v>949.900.896-7</v>
       </c>
       <c r="E99" t="str">
-        <v>604 345 25 96</v>
+        <v>316 204 98 26</v>
       </c>
       <c r="F99" t="str">
-        <v>Transversal 51 # 27 - 93, Buenos Aires, Medellín</v>
+        <v>Diagonal 70 # 34 - 19, Bello, Medellín</v>
       </c>
       <c r="G99" t="str">
-        <v>2927492799</v>
+        <v>3158543131</v>
       </c>
       <c r="H99" t="str">
         <v>Banco Popular</v>
       </c>
       <c r="I99" t="str">
-        <v>17/08/2023</v>
+        <v>15/08/2017</v>
       </c>
       <c r="J99" t="str">
-        <v>lramos</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="100">
@@ -3591,25 +3591,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D100" t="str">
-        <v>961.323.815-9</v>
+        <v>948.911.785-1</v>
       </c>
       <c r="E100" t="str">
-        <v>329 359 64 59</v>
+        <v>321 466 27 88</v>
       </c>
       <c r="F100" t="str">
-        <v>Calle 12 # 32 - 76, Castilla, Medellín</v>
+        <v>Calle 38 # 35 - 62, La América, Medellín</v>
       </c>
       <c r="G100" t="str">
-        <v>3668207859</v>
+        <v>2113248424</v>
       </c>
       <c r="H100" t="str">
-        <v>BBVA Colombia</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I100" t="str">
-        <v>22/01/2021</v>
+        <v>10/04/2018</v>
       </c>
       <c r="J100" t="str">
-        <v>lramos</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="101">
@@ -3623,22 +3623,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D101" t="str">
-        <v>937.516.524-2</v>
+        <v>989.446.512-2</v>
       </c>
       <c r="E101" t="str">
-        <v>309 284 66 81</v>
+        <v>604 437 85 97</v>
       </c>
       <c r="F101" t="str">
-        <v>Avenida 82 # 75 - 35, Girardota, Medellín</v>
+        <v>Transversal 94A # 67 - 61, Laureles, Medellín</v>
       </c>
       <c r="G101" t="str">
-        <v>8390683037</v>
+        <v>7275015188</v>
       </c>
       <c r="H101" t="str">
-        <v>Banco de Occidente</v>
+        <v>Bancolombia</v>
       </c>
       <c r="I101" t="str">
-        <v>28/08/2017</v>
+        <v>15/06/2019</v>
       </c>
       <c r="J101" t="str">
         <v>lramos</v>
@@ -3658,19 +3658,19 @@
         <v/>
       </c>
       <c r="E102" t="str">
-        <v>303 330 45 61</v>
+        <v>326 535 26 22</v>
       </c>
       <c r="F102" t="str">
-        <v>Carrera 52 # 21 - 63, Copacabana, Medellín</v>
+        <v>Calle 75 # 9 - 94, Laureles, Medellín</v>
       </c>
       <c r="G102" t="str">
-        <v>2604562509</v>
+        <v>8550143817</v>
       </c>
       <c r="H102" t="str">
-        <v>Davivienda</v>
+        <v>Banco AV Villas</v>
       </c>
       <c r="I102" t="str">
-        <v>15/06/2020</v>
+        <v>06/07/2023</v>
       </c>
       <c r="J102" t="str">
         <v>dcastro</v>
@@ -3687,22 +3687,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D103" t="str">
-        <v>982.246.304-3</v>
+        <v>965.655.056-4</v>
       </c>
       <c r="E103" t="str">
-        <v>300 523 70 94</v>
+        <v>604 799 39 69</v>
       </c>
       <c r="F103" t="str">
-        <v>Carrera 2 # 72 - 17, Envigado, Medellín</v>
+        <v>Calle 66A # 38 - 48, La Estrella, Medellín</v>
       </c>
       <c r="G103" t="str">
-        <v>6506018841</v>
+        <v>3127809829</v>
       </c>
       <c r="H103" t="str">
-        <v>Scotiabank Colpatria</v>
+        <v>Banco Popular</v>
       </c>
       <c r="I103" t="str">
-        <v>30/04/2020</v>
+        <v>26/07/2018</v>
       </c>
       <c r="J103" t="str">
         <v>lramos</v>
@@ -3719,25 +3719,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D104" t="str">
-        <v>916.476.724-1</v>
+        <v>964.576.832-0</v>
       </c>
       <c r="E104" t="str">
-        <v>604 407 39 50</v>
+        <v>303 588 73 61</v>
       </c>
       <c r="F104" t="str">
-        <v>Calle 32 # 96 - 59, Envigado, Medellín</v>
+        <v>Carrera 45 # 97 - 70, Bello, Medellín</v>
       </c>
       <c r="G104" t="str">
-        <v>8420489439</v>
+        <v>3598021491</v>
       </c>
       <c r="H104" t="str">
         <v>Banco AV Villas</v>
       </c>
       <c r="I104" t="str">
-        <v>05/04/2021</v>
+        <v>18/03/2021</v>
       </c>
       <c r="J104" t="str">
-        <v>dcastro</v>
+        <v>kalzate</v>
       </c>
     </row>
     <row r="105">
@@ -3751,22 +3751,22 @@
         <v>CLIENTE</v>
       </c>
       <c r="D105" t="str">
-        <v>964.952.429-8</v>
+        <v>998.596.788-3</v>
       </c>
       <c r="E105" t="str">
-        <v>318 622 23 52</v>
+        <v>325 796 28 93</v>
       </c>
       <c r="F105" t="str">
-        <v>Avenida 14 # 56 - 29, Castilla, Medellín</v>
+        <v>Carrera 76 # 96 - 44, Caldas, Medellín</v>
       </c>
       <c r="G105" t="str">
-        <v>4784738188</v>
+        <v>7290887196</v>
       </c>
       <c r="H105" t="str">
         <v>Banco Popular</v>
       </c>
       <c r="I105" t="str">
-        <v>19/10/2024</v>
+        <v>04/05/2024</v>
       </c>
       <c r="J105" t="str">
         <v>kalzate</v>
@@ -3783,25 +3783,25 @@
         <v>CLIENTE</v>
       </c>
       <c r="D106" t="str">
-        <v>976.621.586-1</v>
+        <v>992.104.611-7</v>
       </c>
       <c r="E106" t="str">
-        <v>604 414 53 31</v>
+        <v>302 631 68 94</v>
       </c>
       <c r="F106" t="str">
-        <v>Carrera 77 # 69 - 91, Copacabana, Medellín</v>
+        <v>Calle 64 # 44 - 88, Bello, Medellín</v>
       </c>
       <c r="G106" t="str">
-        <v>6856358084</v>
+        <v>5964069054</v>
       </c>
       <c r="H106" t="str">
         <v>Banco de Occidente</v>
       </c>
       <c r="I106" t="str">
-        <v>04/09/2023</v>
+        <v>08/12/2024</v>
       </c>
       <c r="J106" t="str">
-        <v>kalzate</v>
+        <v>lramos</v>
       </c>
     </row>
     <row r="107">
@@ -3815,22 +3815,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D107" t="str">
-        <v>1.065.438.457-0</v>
+        <v>1.071.059.916-5</v>
       </c>
       <c r="E107" t="str">
-        <v>314 681 17 27</v>
+        <v>305 754 35 86</v>
       </c>
       <c r="F107" t="str">
-        <v>Transversal 81 # 96 - 87, Laureles, Medellín</v>
+        <v>Avenida 77A # 41 - 87, Buenos Aires, Medellín</v>
       </c>
       <c r="G107" t="str">
-        <v>1656689443</v>
+        <v>4580749024</v>
       </c>
       <c r="H107" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I107" t="str">
-        <v>12/09/2022</v>
+        <v>21/07/2021</v>
       </c>
       <c r="J107" t="str">
         <v>ncardona</v>
@@ -3847,22 +3847,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D108" t="str">
-        <v>1.079.711.319-3</v>
+        <v>1.005.729.868-5</v>
       </c>
       <c r="E108" t="str">
-        <v>324 669 88 89</v>
+        <v>304 803 78 92</v>
       </c>
       <c r="F108" t="str">
-        <v>Carrera 77 # 6 - 21, Rionegro, Medellín</v>
+        <v>Diagonal 84A # 94 - 41, Aranjuez, Medellín</v>
       </c>
       <c r="G108" t="str">
-        <v>3789269838</v>
+        <v>5998644129</v>
       </c>
       <c r="H108" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I108" t="str">
-        <v>05/06/2022</v>
+        <v>18/01/2023</v>
       </c>
       <c r="J108" t="str">
         <v>ncardona</v>
@@ -3879,22 +3879,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D109" t="str">
-        <v>1.040.387.914-4</v>
+        <v>1.002.099.603-5</v>
       </c>
       <c r="E109" t="str">
-        <v>301 422 26 34</v>
+        <v>305 417 81 31</v>
       </c>
       <c r="F109" t="str">
-        <v>Avenida 57A # 93 - 69, Rionegro, Medellín</v>
+        <v>Diagonal 41A # 37 - 79, La América, Medellín</v>
       </c>
       <c r="G109" t="str">
-        <v>5629666054</v>
+        <v>5998698294</v>
       </c>
       <c r="H109" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I109" t="str">
-        <v>14/02/2021</v>
+        <v>08/05/2020</v>
       </c>
       <c r="J109" t="str">
         <v>ncardona</v>
@@ -3911,13 +3911,13 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D110" t="str">
-        <v>1.044.643.138-8</v>
+        <v>1.017.096.330-0</v>
       </c>
       <c r="E110" t="str">
-        <v>325 319 75 48</v>
+        <v>301 762 67 34</v>
       </c>
       <c r="F110" t="str">
-        <v>Diagonal 60 # 44 - 13, Manrique, Medellín</v>
+        <v>Calle 81 # 93 - 97, Bello, Medellín</v>
       </c>
       <c r="G110" t="str">
         <v>0230456789</v>
@@ -3926,7 +3926,7 @@
         <v>Bancolombia</v>
       </c>
       <c r="I110" t="str">
-        <v>20/06/2020</v>
+        <v>08/06/2022</v>
       </c>
       <c r="J110" t="str">
         <v>ncardona</v>
@@ -3943,22 +3943,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D111" t="str">
-        <v>1.025.158.551-8</v>
+        <v>1.086.062.824-1</v>
       </c>
       <c r="E111" t="str">
-        <v>311 619 98 95</v>
+        <v>322 596 23 59</v>
       </c>
       <c r="F111" t="str">
-        <v>Transversal 31 # 11 - 26, Copacabana, Medellín</v>
+        <v>Transversal 7 # 8 - 20, Laureles, Medellín</v>
       </c>
       <c r="G111" t="str">
-        <v>8860886333</v>
+        <v>9918461352</v>
       </c>
       <c r="H111" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I111" t="str">
-        <v>04/02/2022</v>
+        <v>31/05/2020</v>
       </c>
       <c r="J111" t="str">
         <v>ncardona</v>
@@ -3975,22 +3975,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D112" t="str">
-        <v>1.057.976.935-8</v>
+        <v>1.023.694.821-2</v>
       </c>
       <c r="E112" t="str">
-        <v>320 809 88 28</v>
+        <v>316 557 55 85</v>
       </c>
       <c r="F112" t="str">
-        <v>Avenida 42A # 36 - 78, Castilla, Medellín</v>
+        <v>Calle 96 # 9 - 30, Envigado, Medellín</v>
       </c>
       <c r="G112" t="str">
-        <v>1628928801</v>
+        <v>9512690083</v>
       </c>
       <c r="H112" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I112" t="str">
-        <v>28/01/2022</v>
+        <v>14/10/2021</v>
       </c>
       <c r="J112" t="str">
         <v>ncardona</v>
@@ -4007,22 +4007,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D113" t="str">
-        <v>1.013.493.175-3</v>
+        <v>1.062.817.660-5</v>
       </c>
       <c r="E113" t="str">
-        <v>303 250 58 44</v>
+        <v>321 729 98 31</v>
       </c>
       <c r="F113" t="str">
-        <v>Transversal 44 # 62 - 38, Envigado, Medellín</v>
+        <v>Avenida 31 # 21 - 54, Manrique, Medellín</v>
       </c>
       <c r="G113" t="str">
-        <v>9429325902</v>
+        <v>3125752614</v>
       </c>
       <c r="H113" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I113" t="str">
-        <v>12/11/2020</v>
+        <v>27/07/2022</v>
       </c>
       <c r="J113" t="str">
         <v>ncardona</v>
@@ -4039,22 +4039,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D114" t="str">
-        <v>1.002.698.488-4</v>
+        <v>1.083.289.626-4</v>
       </c>
       <c r="E114" t="str">
-        <v>302 583 14 44</v>
+        <v>328 386 17 59</v>
       </c>
       <c r="F114" t="str">
-        <v>Diagonal 43 # 45 - 17, Manrique, Medellín</v>
+        <v>Avenida 37 # 13 - 99, Girardota, Medellín</v>
       </c>
       <c r="G114" t="str">
-        <v>1175221575</v>
+        <v>8443897523</v>
       </c>
       <c r="H114" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I114" t="str">
-        <v>28/07/2021</v>
+        <v>14/05/2023</v>
       </c>
       <c r="J114" t="str">
         <v>ncardona</v>
@@ -4071,22 +4071,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D115" t="str">
-        <v>1.064.706.024-1</v>
+        <v>1.090.674.302-1</v>
       </c>
       <c r="E115" t="str">
-        <v>318 794 59 14</v>
+        <v>326 604 49 27</v>
       </c>
       <c r="F115" t="str">
-        <v>Calle 41A # 39 - 74, Copacabana, Medellín</v>
+        <v>Diagonal 25 # 87 - 75, Itagüí, Medellín</v>
       </c>
       <c r="G115" t="str">
-        <v>1344697603</v>
+        <v>4409082925</v>
       </c>
       <c r="H115" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I115" t="str">
-        <v>16/03/2023</v>
+        <v>07/10/2018</v>
       </c>
       <c r="J115" t="str">
         <v>ncardona</v>
@@ -4103,22 +4103,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D116" t="str">
-        <v>1.082.634.085-6</v>
+        <v>1.044.600.563-0</v>
       </c>
       <c r="E116" t="str">
-        <v>316 666 17 85</v>
+        <v>302 519 36 21</v>
       </c>
       <c r="F116" t="str">
-        <v>Avenida 91 # 9 - 99, Girardota, Medellín</v>
+        <v>Diagonal 85 # 46 - 28, Manrique, Medellín</v>
       </c>
       <c r="G116" t="str">
-        <v>3821438038</v>
+        <v>5428744623</v>
       </c>
       <c r="H116" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I116" t="str">
-        <v>16/02/2022</v>
+        <v>10/07/2022</v>
       </c>
       <c r="J116" t="str">
         <v>ncardona</v>
@@ -4135,22 +4135,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D117" t="str">
-        <v>1.058.387.929-1</v>
+        <v>1.060.006.941-2</v>
       </c>
       <c r="E117" t="str">
-        <v>328 834 37 79</v>
+        <v>303 824 24 85</v>
       </c>
       <c r="F117" t="str">
-        <v>Transversal 86 # 71 - 65, Castilla, Medellín</v>
+        <v>Carrera 61 # 24 - 33, Buenos Aires, Medellín</v>
       </c>
       <c r="G117" t="str">
-        <v>1333784008</v>
+        <v>5613730795</v>
       </c>
       <c r="H117" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I117" t="str">
-        <v>10/04/2019</v>
+        <v>31/01/2021</v>
       </c>
       <c r="J117" t="str">
         <v>ncardona</v>
@@ -4167,22 +4167,22 @@
         <v>EMPLEADO</v>
       </c>
       <c r="D118" t="str">
-        <v>1.049.122.115-1</v>
+        <v>1.062.702.972-3</v>
       </c>
       <c r="E118" t="str">
-        <v>329 318 12 42</v>
+        <v>327 437 53 91</v>
       </c>
       <c r="F118" t="str">
-        <v>Calle 16 # 32 - 67, El Poblado, Medellín</v>
+        <v>Calle 79 # 49 - 74, Envigado, Medellín</v>
       </c>
       <c r="G118" t="str">
-        <v>7883734154</v>
+        <v>6470498068</v>
       </c>
       <c r="H118" t="str">
         <v>Bancolombia</v>
       </c>
       <c r="I118" t="str">
-        <v>11/03/2019</v>
+        <v>24/07/2019</v>
       </c>
       <c r="J118" t="str">
         <v>ncardona</v>
@@ -4229,39 +4229,39 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CLI-044</v>
+        <v>EMP-10</v>
       </c>
       <c r="B2" t="str">
-        <v>CUENTA BANCARIA</v>
+        <v>TELEFONO</v>
       </c>
       <c r="C2" t="str">
-        <v>4778079589</v>
+        <v>305 235 44 64</v>
       </c>
       <c r="D2" t="str">
-        <v>4784738188</v>
+        <v>302 519 36 21</v>
       </c>
       <c r="E2" t="str">
-        <v>25/03/2025</v>
+        <v>24/03/2025</v>
       </c>
       <c r="F2" t="str">
-        <v>jvargas</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP-06</v>
+        <v>PRV-012</v>
       </c>
       <c r="B3" t="str">
-        <v>TELEFONO</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C3" t="str">
-        <v>321 550 58 62</v>
+        <v>Transversal 68 # 67 - 94, Envigado, Medellín</v>
       </c>
       <c r="D3" t="str">
-        <v>320 809 88 28</v>
+        <v>Avenida 36 # 79 - 93, La Estrella, Medellín</v>
       </c>
       <c r="E3" t="str">
-        <v>28/03/2025</v>
+        <v>21/04/2025</v>
       </c>
       <c r="F3" t="str">
         <v>ncardona</v>
@@ -4269,39 +4269,39 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CLI-014</v>
+        <v>PRV-042</v>
       </c>
       <c r="B4" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C4" t="str">
-        <v>327 413 51 75</v>
+        <v>604 714 23 40</v>
       </c>
       <c r="D4" t="str">
-        <v>314 427 30 53</v>
+        <v>604 730 51 28</v>
       </c>
       <c r="E4" t="str">
-        <v>05/05/2025</v>
+        <v>22/04/2025</v>
       </c>
       <c r="F4" t="str">
-        <v>lramos</v>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CLI-017</v>
+        <v>PRV-006</v>
       </c>
       <c r="B5" t="str">
-        <v>CUENTA BANCARIA</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C5" t="str">
-        <v>1265027899</v>
+        <v>Calle 81 # 67 - 22, Belén, Medellín</v>
       </c>
       <c r="D5" t="str">
-        <v>8221903263</v>
+        <v>Avenida 58 # 33 - 69, Caldas, Medellín</v>
       </c>
       <c r="E5" t="str">
-        <v>07/05/2025</v>
+        <v>28/04/2025</v>
       </c>
       <c r="F5" t="str">
         <v>ncardona</v>
@@ -4309,19 +4309,19 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EMP-03</v>
+        <v>PRV-003</v>
       </c>
       <c r="B6" t="str">
         <v>DIRECCION</v>
       </c>
       <c r="C6" t="str">
-        <v>Carrera 21A # 13 - 49, Copacabana, Medellín</v>
+        <v>Avenida 16 # 17 - 61, El Poblado, Medellín</v>
       </c>
       <c r="D6" t="str">
-        <v>Avenida 57A # 93 - 69, Rionegro, Medellín</v>
+        <v>Avenida 95 # 95 - 30, San Javier, Medellín</v>
       </c>
       <c r="E6" t="str">
-        <v>03/06/2025</v>
+        <v>05/05/2025</v>
       </c>
       <c r="F6" t="str">
         <v>ncardona</v>
@@ -4329,19 +4329,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EMP-07</v>
+        <v>CLI-023</v>
       </c>
       <c r="B7" t="str">
         <v>DIRECCION</v>
       </c>
       <c r="C7" t="str">
-        <v>Diagonal 92 # 18 - 33, Laureles, Medellín</v>
+        <v>Calle 27 # 22 - 63, Robledo, Medellín</v>
       </c>
       <c r="D7" t="str">
-        <v>Transversal 44 # 62 - 38, Envigado, Medellín</v>
+        <v>Carrera 37 # 93 - 91, Buenos Aires, Medellín</v>
       </c>
       <c r="E7" t="str">
-        <v>11/06/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="F7" t="str">
         <v>ncardona</v>
@@ -4349,39 +4349,39 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CLI-002</v>
+        <v>PRV-018</v>
       </c>
       <c r="B8" t="str">
-        <v>CUENTA BANCARIA</v>
+        <v>TELEFONO</v>
       </c>
       <c r="C8" t="str">
-        <v>7240787432</v>
+        <v>604 341 13 28</v>
       </c>
       <c r="D8" t="str">
-        <v>6809769989</v>
+        <v>604 528 52 39</v>
       </c>
       <c r="E8" t="str">
-        <v>25/06/2025</v>
+        <v>03/06/2025</v>
       </c>
       <c r="F8" t="str">
-        <v>lramos</v>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PRV-009</v>
+        <v>PRV-021</v>
       </c>
       <c r="B9" t="str">
-        <v>TELEFONO</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C9" t="str">
-        <v>604 689 87 51</v>
+        <v>Transversal 51 # 27 - 93, Buenos Aires, Medellín</v>
       </c>
       <c r="D9" t="str">
-        <v>604 734 91 84</v>
+        <v>Calle 76 # 41 - 33, Belén, Medellín</v>
       </c>
       <c r="E9" t="str">
-        <v>01/07/2025</v>
+        <v>09/06/2025</v>
       </c>
       <c r="F9" t="str">
         <v>mosorio</v>
@@ -4389,19 +4389,19 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>PRV-039</v>
+        <v>CLI-002</v>
       </c>
       <c r="B10" t="str">
-        <v>DIRECCION</v>
+        <v>CUENTA BANCARIA</v>
       </c>
       <c r="C10" t="str">
-        <v>Transversal 3 # 46 - 95, Aranjuez, Medellín</v>
+        <v>6319765105</v>
       </c>
       <c r="D10" t="str">
-        <v>Avenida 84 # 13 - 37, La Estrella, Medellín</v>
+        <v>7402971211</v>
       </c>
       <c r="E10" t="str">
-        <v>21/07/2025</v>
+        <v>16/06/2025</v>
       </c>
       <c r="F10" t="str">
         <v>ncardona</v>
@@ -4409,39 +4409,39 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>PRV-036</v>
+        <v>CLI-005</v>
       </c>
       <c r="B11" t="str">
-        <v>TELEFONO</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C11" t="str">
-        <v>604 287 19 77</v>
+        <v>Calle 55 # 16 - 48, Robledo, Medellín</v>
       </c>
       <c r="D11" t="str">
-        <v>604 708 92 81</v>
+        <v>Carrera 33 # 61 - 42, La Estrella, Medellín</v>
       </c>
       <c r="E11" t="str">
-        <v>19/08/2025</v>
+        <v>25/06/2025</v>
       </c>
       <c r="F11" t="str">
-        <v>mosorio</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CLI-041</v>
+        <v>PRV-027</v>
       </c>
       <c r="B12" t="str">
         <v>DIRECCION</v>
       </c>
       <c r="C12" t="str">
-        <v>Calle 74 # 45 - 72, San Javier, Medellín</v>
+        <v>Transversal 9A # 45 - 39, San Javier, Medellín</v>
       </c>
       <c r="D12" t="str">
-        <v>Carrera 52 # 21 - 63, Copacabana, Medellín</v>
+        <v>Calle 37 # 16 - 19, Bello, Medellín</v>
       </c>
       <c r="E12" t="str">
-        <v>22/08/2025</v>
+        <v>07/07/2025</v>
       </c>
       <c r="F12" t="str">
         <v>ncardona</v>
@@ -4449,59 +4449,59 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>EMP-04</v>
+        <v>CLI-041</v>
       </c>
       <c r="B13" t="str">
         <v>DIRECCION</v>
       </c>
       <c r="C13" t="str">
-        <v>Carrera 68 # 17 - 84, Aranjuez, Medellín</v>
+        <v>Diagonal 40A # 20 - 38, Guayabal, Medellín</v>
       </c>
       <c r="D13" t="str">
-        <v>Diagonal 60 # 44 - 13, Manrique, Medellín</v>
+        <v>Calle 75 # 9 - 94, Laureles, Medellín</v>
       </c>
       <c r="E13" t="str">
-        <v>01/09/2025</v>
+        <v>22/07/2025</v>
       </c>
       <c r="F13" t="str">
-        <v>ncardona</v>
+        <v>jvargas</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CLI-038</v>
+        <v>PRV-030</v>
       </c>
       <c r="B14" t="str">
         <v>DIRECCION</v>
       </c>
       <c r="C14" t="str">
-        <v>Transversal 37 # 7 - 16, El Poblado, Medellín</v>
+        <v>Avenida 36 # 13 - 43, Rionegro, Medellín</v>
       </c>
       <c r="D14" t="str">
-        <v>Transversal 51 # 27 - 93, Buenos Aires, Medellín</v>
+        <v>Avenida 11 # 50 - 40, San Javier, Medellín</v>
       </c>
       <c r="E14" t="str">
-        <v>15/09/2025</v>
+        <v>23/07/2025</v>
       </c>
       <c r="F14" t="str">
-        <v>ncardona</v>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>EMP-09</v>
+        <v>CLI-017</v>
       </c>
       <c r="B15" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C15" t="str">
-        <v>309 320 11 85</v>
+        <v>309 872 59 30</v>
       </c>
       <c r="D15" t="str">
-        <v>318 794 59 14</v>
+        <v>300 842 71 83</v>
       </c>
       <c r="E15" t="str">
-        <v>03/10/2025</v>
+        <v>25/08/2025</v>
       </c>
       <c r="F15" t="str">
         <v>ncardona</v>
@@ -4509,79 +4509,79 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>PRV-006</v>
+        <v>CLI-011</v>
       </c>
       <c r="B16" t="str">
-        <v>TELEFONO</v>
+        <v>CUENTA BANCARIA</v>
       </c>
       <c r="C16" t="str">
-        <v>604 879 46 65</v>
+        <v>7754385490</v>
       </c>
       <c r="D16" t="str">
-        <v>604 667 55 40</v>
+        <v>1658526075</v>
       </c>
       <c r="E16" t="str">
-        <v>06/10/2025</v>
+        <v>08/09/2025</v>
       </c>
       <c r="F16" t="str">
-        <v>mosorio</v>
+        <v>jvargas</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>PRV-033</v>
+        <v>CLI-020</v>
       </c>
       <c r="B17" t="str">
-        <v>TELEFONO</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C17" t="str">
-        <v>604 468 90 88</v>
+        <v>Transversal 56 # 72 - 47, Caldas, Medellín</v>
       </c>
       <c r="D17" t="str">
-        <v>604 209 96 40</v>
+        <v>Diagonal 39 # 34 - 59, Sabaneta, Medellín</v>
       </c>
       <c r="E17" t="str">
-        <v>14/10/2025</v>
+        <v>08/09/2025</v>
       </c>
       <c r="F17" t="str">
-        <v>mosorio</v>
+        <v>lramos</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>PRV-024</v>
+        <v>EMP-08</v>
       </c>
       <c r="B18" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C18" t="str">
-        <v>604 402 14 46</v>
+        <v>313 482 50 34</v>
       </c>
       <c r="D18" t="str">
-        <v>604 638 17 70</v>
+        <v>328 386 17 59</v>
       </c>
       <c r="E18" t="str">
-        <v>17/10/2025</v>
+        <v>15/09/2025</v>
       </c>
       <c r="F18" t="str">
-        <v>mosorio</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>EMP-08</v>
+        <v>CLI-038</v>
       </c>
       <c r="B19" t="str">
-        <v>TELEFONO</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C19" t="str">
-        <v>306 231 78 11</v>
+        <v>Avenida 39 # 33 - 15, Belén, Medellín</v>
       </c>
       <c r="D19" t="str">
-        <v>302 583 14 44</v>
+        <v>Diagonal 70 # 34 - 19, Bello, Medellín</v>
       </c>
       <c r="E19" t="str">
-        <v>20/10/2025</v>
+        <v>14/10/2025</v>
       </c>
       <c r="F19" t="str">
         <v>ncardona</v>
@@ -4589,119 +4589,119 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>PRV-042</v>
+        <v>EMP-01</v>
       </c>
       <c r="B20" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C20" t="str">
-        <v>604 231 23 93</v>
+        <v>325 319 75 48</v>
       </c>
       <c r="D20" t="str">
-        <v>604 406 83 90</v>
+        <v>305 754 35 86</v>
       </c>
       <c r="E20" t="str">
-        <v>24/10/2025</v>
+        <v>05/11/2025</v>
       </c>
       <c r="F20" t="str">
-        <v>mosorio</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CLI-035</v>
+        <v>EMP-03</v>
       </c>
       <c r="B21" t="str">
-        <v>CUENTA BANCARIA</v>
+        <v>TELEFONO</v>
       </c>
       <c r="C21" t="str">
-        <v>4205094014</v>
+        <v>303 332 63 98</v>
       </c>
       <c r="D21" t="str">
-        <v>2552438711</v>
+        <v>305 417 81 31</v>
       </c>
       <c r="E21" t="str">
-        <v>30/10/2025</v>
+        <v>22/12/2025</v>
       </c>
       <c r="F21" t="str">
-        <v>jvargas</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CLI-011</v>
+        <v>EMP-07</v>
       </c>
       <c r="B22" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C22" t="str">
-        <v>300 412 69 44</v>
+        <v>311 629 22 29</v>
       </c>
       <c r="D22" t="str">
-        <v>327 749 71 93</v>
+        <v>321 729 98 31</v>
       </c>
       <c r="E22" t="str">
-        <v>13/11/2025</v>
+        <v>29/12/2025</v>
       </c>
       <c r="F22" t="str">
-        <v>lramos</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>EMP-01</v>
+        <v>PRV-009</v>
       </c>
       <c r="B23" t="str">
         <v>DIRECCION</v>
       </c>
       <c r="C23" t="str">
-        <v>Carrera 55 # 7 - 70, San Javier, Medellín</v>
+        <v>Avenida 54 # 74 - 70, La Estrella, Medellín</v>
       </c>
       <c r="D23" t="str">
-        <v>Transversal 81 # 96 - 87, Laureles, Medellín</v>
+        <v>Carrera 21 # 99 - 44, Manrique, Medellín</v>
       </c>
       <c r="E23" t="str">
-        <v>20/11/2025</v>
+        <v>06/01/2026</v>
       </c>
       <c r="F23" t="str">
-        <v>ncardona</v>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>PRV-021</v>
+        <v>CLI-014</v>
       </c>
       <c r="B24" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C24" t="str">
-        <v>604 835 49 36</v>
+        <v>324 384 24 36</v>
       </c>
       <c r="D24" t="str">
-        <v>604 203 88 46</v>
+        <v>322 574 78 47</v>
       </c>
       <c r="E24" t="str">
-        <v>01/12/2025</v>
+        <v>20/01/2026</v>
       </c>
       <c r="F24" t="str">
-        <v>mosorio</v>
+        <v>jvargas</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>EMP-02</v>
+        <v>EMP-09</v>
       </c>
       <c r="B25" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C25" t="str">
-        <v>320 582 81 21</v>
+        <v>309 456 29 48</v>
       </c>
       <c r="D25" t="str">
-        <v>324 669 88 89</v>
+        <v>326 604 49 27</v>
       </c>
       <c r="E25" t="str">
-        <v>03/12/2025</v>
+        <v>21/01/2026</v>
       </c>
       <c r="F25" t="str">
         <v>ncardona</v>
@@ -4709,19 +4709,19 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>CLI-023</v>
+        <v>CLI-008</v>
       </c>
       <c r="B26" t="str">
         <v>CUENTA BANCARIA</v>
       </c>
       <c r="C26" t="str">
-        <v>8898716703</v>
+        <v>1515649246</v>
       </c>
       <c r="D26" t="str">
-        <v>3296848016</v>
+        <v>7325122768</v>
       </c>
       <c r="E26" t="str">
-        <v>10/12/2025</v>
+        <v>23/02/2026</v>
       </c>
       <c r="F26" t="str">
         <v>ncardona</v>
@@ -4729,19 +4729,19 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>CLI-029</v>
+        <v>EMP-02</v>
       </c>
       <c r="B27" t="str">
-        <v>CUENTA BANCARIA</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C27" t="str">
-        <v>4372159245</v>
+        <v>Diagonal 44A # 66 - 13, Rionegro, Medellín</v>
       </c>
       <c r="D27" t="str">
-        <v>1308440032</v>
+        <v>Diagonal 84A # 94 - 41, Aranjuez, Medellín</v>
       </c>
       <c r="E27" t="str">
-        <v>13/01/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="F27" t="str">
         <v>ncardona</v>
@@ -4749,59 +4749,59 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>CLI-032</v>
+        <v>CLI-029</v>
       </c>
       <c r="B28" t="str">
-        <v>CUENTA BANCARIA</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C28" t="str">
-        <v>2806247459</v>
+        <v>Avenida 76 # 84 - 48, Robledo, Medellín</v>
       </c>
       <c r="D28" t="str">
-        <v>5199349244</v>
+        <v>Transversal 15A # 49 - 37, Bello, Medellín</v>
       </c>
       <c r="E28" t="str">
-        <v>13/01/2026</v>
+        <v>13/04/2026</v>
       </c>
       <c r="F28" t="str">
-        <v>jvargas</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>EMP-10</v>
+        <v>PRV-039</v>
       </c>
       <c r="B29" t="str">
-        <v>DIRECCION</v>
+        <v>TELEFONO</v>
       </c>
       <c r="C29" t="str">
-        <v>Transversal 16 # 32 - 22, Guayabal, Medellín</v>
+        <v>604 717 54 16</v>
       </c>
       <c r="D29" t="str">
-        <v>Avenida 91 # 9 - 99, Girardota, Medellín</v>
+        <v>604 700 77 18</v>
       </c>
       <c r="E29" t="str">
-        <v>13/01/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="F29" t="str">
-        <v>ncardona</v>
+        <v>mosorio</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>PRV-003</v>
+        <v>PRV-036</v>
       </c>
       <c r="B30" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C30" t="str">
-        <v>604 757 81 96</v>
+        <v>604 728 35 93</v>
       </c>
       <c r="D30" t="str">
-        <v>604 681 23 19</v>
+        <v>604 340 33 91</v>
       </c>
       <c r="E30" t="str">
-        <v>13/01/2026</v>
+        <v>11/05/2026</v>
       </c>
       <c r="F30" t="str">
         <v>mosorio</v>
@@ -4809,59 +4809,59 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>PRV-030</v>
+        <v>EMP-05</v>
       </c>
       <c r="B31" t="str">
-        <v>DIRECCION</v>
+        <v>TELEFONO</v>
       </c>
       <c r="C31" t="str">
-        <v>Avenida 79A # 24 - 75, La Estrella, Medellín</v>
+        <v>315 870 16 88</v>
       </c>
       <c r="D31" t="str">
-        <v>Carrera 49 # 66 - 41, La América, Medellín</v>
+        <v>322 596 23 59</v>
       </c>
       <c r="E31" t="str">
-        <v>26/01/2026</v>
+        <v>19/05/2026</v>
       </c>
       <c r="F31" t="str">
-        <v>mosorio</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>CLI-020</v>
+        <v>CLI-044</v>
       </c>
       <c r="B32" t="str">
-        <v>DIRECCION</v>
+        <v>TELEFONO</v>
       </c>
       <c r="C32" t="str">
-        <v>Transversal 50 # 49 - 85, Girardota, Medellín</v>
+        <v>326 875 53 62</v>
       </c>
       <c r="D32" t="str">
-        <v>Avenida 34 # 46 - 87, Sabaneta, Medellín</v>
+        <v>325 796 28 93</v>
       </c>
       <c r="E32" t="str">
-        <v>09/02/2026</v>
+        <v>25/05/2026</v>
       </c>
       <c r="F32" t="str">
-        <v>ncardona</v>
+        <v>lramos</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>CLI-005</v>
+        <v>PRV-015</v>
       </c>
       <c r="B33" t="str">
-        <v>CUENTA BANCARIA</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C33" t="str">
-        <v>7857461324</v>
+        <v>Carrera 40 # 68 - 70, Castilla, Medellín</v>
       </c>
       <c r="D33" t="str">
-        <v>4294175456</v>
+        <v>Calle 64 # 64 - 77, El Poblado, Medellín</v>
       </c>
       <c r="E33" t="str">
-        <v>30/03/2026</v>
+        <v>25/05/2026</v>
       </c>
       <c r="F33" t="str">
         <v>ncardona</v>
@@ -4872,39 +4872,39 @@
         <v>CLI-026</v>
       </c>
       <c r="B34" t="str">
-        <v>TELEFONO</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C34" t="str">
-        <v>315 745 10 28</v>
+        <v>Diagonal 76A # 31 - 53, Envigado, Medellín</v>
       </c>
       <c r="D34" t="str">
-        <v>604 650 59 99</v>
+        <v>Calle 26 # 59 - 84, Sabaneta, Medellín</v>
       </c>
       <c r="E34" t="str">
-        <v>30/03/2026</v>
+        <v>28/05/2026</v>
       </c>
       <c r="F34" t="str">
-        <v>lramos</v>
+        <v>jvargas</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>PRV-018</v>
+        <v>EMP-06</v>
       </c>
       <c r="B35" t="str">
-        <v>DIRECCION</v>
+        <v>TELEFONO</v>
       </c>
       <c r="C35" t="str">
-        <v>Diagonal 51 # 79 - 76, Caldas, Medellín</v>
+        <v>324 207 41 78</v>
       </c>
       <c r="D35" t="str">
-        <v>Calle 90 # 87 - 95, La Estrella, Medellín</v>
+        <v>316 557 55 85</v>
       </c>
       <c r="E35" t="str">
-        <v>08/04/2026</v>
+        <v>01/06/2026</v>
       </c>
       <c r="F35" t="str">
-        <v>mosorio</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="36">
@@ -4915,7 +4915,7 @@
         <v>CUENTA BANCARIA</v>
       </c>
       <c r="C36" t="str">
-        <v>6620685945</v>
+        <v>8414377484</v>
       </c>
       <c r="D36" t="str">
         <v>8801234455</v>
@@ -4929,19 +4929,19 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>EMP-05</v>
+        <v>PRV-024</v>
       </c>
       <c r="B37" t="str">
-        <v>TELEFONO</v>
+        <v>DIRECCION</v>
       </c>
       <c r="C37" t="str">
-        <v>320 504 22 21</v>
+        <v>Diagonal 81A # 61 - 97, Girardota, Medellín</v>
       </c>
       <c r="D37" t="str">
-        <v>311 619 98 95</v>
+        <v>Calle 25 # 63 - 98, Laureles, Medellín</v>
       </c>
       <c r="E37" t="str">
-        <v>30/06/2026</v>
+        <v>23/06/2026</v>
       </c>
       <c r="F37" t="str">
         <v>ncardona</v>
@@ -4949,19 +4949,19 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>PRV-027</v>
+        <v>EMP-04</v>
       </c>
       <c r="B38" t="str">
         <v>DIRECCION</v>
       </c>
       <c r="C38" t="str">
-        <v>Diagonal 62A # 56 - 40, La Estrella, Medellín</v>
+        <v>Carrera 86A # 19 - 78, Caldas, Medellín</v>
       </c>
       <c r="D38" t="str">
-        <v>Carrera 47 # 45 - 83, Robledo, Medellín</v>
+        <v>Calle 81 # 93 - 97, Bello, Medellín</v>
       </c>
       <c r="E38" t="str">
-        <v>06/07/2026</v>
+        <v>09/07/2026</v>
       </c>
       <c r="F38" t="str">
         <v>ncardona</v>
@@ -4969,39 +4969,39 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>PRV-012</v>
+        <v>CLI-035</v>
       </c>
       <c r="B39" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C39" t="str">
-        <v>604 886 29 60</v>
+        <v>306 438 73 81</v>
       </c>
       <c r="D39" t="str">
-        <v>604 250 77 68</v>
+        <v>320 594 71 83</v>
       </c>
       <c r="E39" t="str">
-        <v>21/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="F39" t="str">
-        <v>mosorio</v>
+        <v>ncardona</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>PRV-015</v>
+        <v>CLI-032</v>
       </c>
       <c r="B40" t="str">
         <v>DIRECCION</v>
       </c>
       <c r="C40" t="str">
-        <v>Transversal 71 # 85 - 15, Rionegro, Medellín</v>
+        <v>Transversal 68A # 20 - 61, La Estrella, Medellín</v>
       </c>
       <c r="D40" t="str">
-        <v>Transversal 32 # 48 - 60, Girardota, Medellín</v>
+        <v>Calle 68 # 75 - 78, Copacabana, Medellín</v>
       </c>
       <c r="E40" t="str">
-        <v>27/07/2026</v>
+        <v>03/08/2026</v>
       </c>
       <c r="F40" t="str">
         <v>ncardona</v>
@@ -5009,22 +5009,22 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>CLI-008</v>
+        <v>PRV-033</v>
       </c>
       <c r="B41" t="str">
         <v>TELEFONO</v>
       </c>
       <c r="C41" t="str">
-        <v>307 857 64 24</v>
+        <v>604 637 81 96</v>
       </c>
       <c r="D41" t="str">
-        <v>324 304 30 54</v>
+        <v>604 648 53 15</v>
       </c>
       <c r="E41" t="str">
-        <v>31/07/2026</v>
+        <v>03/08/2026</v>
       </c>
       <c r="F41" t="str">
-        <v>ncardona</v>
+        <v>mosorio</v>
       </c>
     </row>
   </sheetData>

</xml_diff>